<commit_message>
Results workbook: Task 3 with the last two A16 reruns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/results/experiment-a-results.xlsx
+++ b/docs/results/experiment-a-results.xlsx
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3115" uniqueCount="803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3155" uniqueCount="813">
   <si>
     <t xml:space="preserve">Experiment results workbook</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated: 2026-10-20T04:18:40Z</t>
+    <t xml:space="preserve">Generated: 2026-10-20T05:40Z</t>
   </si>
   <si>
     <t xml:space="preserve">Runs directory: /workspace/agent-experiments-matrix</t>
@@ -33,13 +33,13 @@
     <t xml:space="preserve">Cost scenario: billed (all USD columns). Claude USD and Codex USD split the scenario's per-model cost; models whose name starts with gpt are Codex, all others are Claude.</t>
   </si>
   <si>
-    <t xml:space="preserve">Superseded runs excluded using: docs/results/superseded.json (26 listed)</t>
+    <t xml:space="preserve">Superseded runs excluded using: docs/results/superseded.json (28 listed)</t>
   </si>
   <si>
     <t xml:space="preserve">Statuses dropped: cli_error, running, stopped, usage_limit</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 25 of 51 attempts in the results</t>
+    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 29 of 59 attempts in the results</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -2130,222 +2130,234 @@
     <t xml:space="preserve">386a4084</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A16 task3 rep 6: lost a round to the ambiguous fresh-event rule and its misleading feedback; rerun on the corrected pack as 731b7bc2</t>
+  </si>
+  <si>
     <t xml:space="preserve">731b7bc2</t>
   </si>
   <si>
+    <t xml:space="preserve">8a759a54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">superseded: A16 task3 rep 7: lost a round to the ambiguous fresh-event rule and its misleading feedback; rerun on the corrected pack as a1fa4a9e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a1fa4a9e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09a3708e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5a50bf47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d27443ac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1ee9f10d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">79ec6f5d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5f80fe5a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a8329bee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ddba0caf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8fe57108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">441f0349</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d43fbb41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19a7c17b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">175d21e1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b76a9d09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00194f35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">433e067c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">58f5b501</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78051b57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f259022b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85c15f29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">506385ff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90812944</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c0df5067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3941ef9b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f1cc8bc8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01dd7930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">403fc948</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7d4be958</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5457d5ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ef1bbeb0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19781877</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fffc24ac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7dde7b16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">df2da5d9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d30af6eb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e77f9343</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b84c3e90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2f6bd8eb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">claude reported an error in round 1 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">357ee0e9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">claude reported an error in round 2 (exit 1): You've hit your session limit · resets 12am (America/Chicago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a203ac20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dfd2359b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0df855ac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2e788e29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">claude reported an error in round 2 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5f946635</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stopped by the owner in round 2: task4 is being redone on a corrected acceptance pack; not a result.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e34260cb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52d7d848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76771788</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5af65ea5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4dbd1845</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59986a93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92450aa4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">claude reported an error in round 3 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d3623279</t>
+  </si>
+  <si>
+    <t xml:space="preserve">claude reported an error in round 3 (exit 1): You've hit your session limit · resets 9:40am (America/Chicago)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66f31f60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98cbe722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d4891735</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fbc44c56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">016ca93e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01e97c9f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f6294287</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c77fc1a9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de4fc384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ee0e6aeb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f305c31e</t>
+  </si>
+  <si>
     <t xml:space="preserve">running</t>
   </si>
   <si>
     <t xml:space="preserve">dropped status: running</t>
   </si>
   <si>
-    <t xml:space="preserve">8a759a54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a1fa4a9e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09a3708e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5a50bf47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d27443ac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1ee9f10d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">79ec6f5d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5f80fe5a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a8329bee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ddba0caf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8fe57108</t>
-  </si>
-  <si>
-    <t xml:space="preserve">441f0349</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d43fbb41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19a7c17b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">175d21e1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b76a9d09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00194f35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">433e067c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">58f5b501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">78051b57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f259022b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">85c15f29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">506385ff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">90812944</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c0df5067</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3941ef9b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f1cc8bc8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01dd7930</t>
-  </si>
-  <si>
-    <t xml:space="preserve">403fc948</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7d4be958</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5457d5ba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ef1bbeb0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19781877</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fffc24ac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7dde7b16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">df2da5d9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d30af6eb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e77f9343</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b84c3e90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2f6bd8eb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">claude reported an error in round 1 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">357ee0e9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">claude reported an error in round 2 (exit 1): You've hit your session limit · resets 12am (America/Chicago)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a203ac20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dfd2359b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0df855ac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2e788e29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">claude reported an error in round 2 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5f946635</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stopped by the owner in round 2: task4 is being redone on a corrected acceptance pack; not a result.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e34260cb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52d7d848</t>
-  </si>
-  <si>
-    <t xml:space="preserve">76771788</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5af65ea5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4dbd1845</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59986a93</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92450aa4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">claude reported an error in round 3 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d3623279</t>
-  </si>
-  <si>
-    <t xml:space="preserve">claude reported an error in round 3 (exit 1): You've hit your session limit · resets 9:40am (America/Chicago)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">66f31f60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">98cbe722</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d4891735</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fbc44c56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">016ca93e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f6294287</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c77fc1a9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">de4fc384</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ee0e6aeb</t>
-  </si>
-  <si>
     <t xml:space="preserve">dd4497e8</t>
   </si>
   <si>
@@ -2370,6 +2382,9 @@
     <t xml:space="preserve">claude reported an error in round 5 (exit 1): You've hit your session limit · resets 6:50pm (America/Chicago)</t>
   </si>
   <si>
+    <t xml:space="preserve">42f0528f</t>
+  </si>
+  <si>
     <t xml:space="preserve">65d92f15</t>
   </si>
   <si>
@@ -2379,6 +2394,9 @@
     <t xml:space="preserve">6536e57a</t>
   </si>
   <si>
+    <t xml:space="preserve">e8c4f691</t>
+  </si>
+  <si>
     <t xml:space="preserve">7137e856</t>
   </si>
   <si>
@@ -2428,6 +2446,18 @@
   </si>
   <si>
     <t xml:space="preserve">a5775bc0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1dbd8ee4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34c1b008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">019d4e30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02411e1d</t>
   </si>
 </sst>
 </file>
@@ -2701,8 +2731,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC10" totalsRowShown="0">
-  <autoFilter ref="A1:AC10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC12" totalsRowShown="0">
+  <autoFilter ref="A1:AC12"/>
   <tableColumns count="29">
     <tableColumn id="1" name="Arm"/>
     <tableColumn id="2" name="Description"/>
@@ -2739,8 +2769,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Runs_T4" displayName="Runs_T4" ref="A1:Z52" totalsRowShown="0">
-  <autoFilter ref="A1:Z52"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Runs_T4" displayName="Runs_T4" ref="A1:Z60" totalsRowShown="0">
+  <autoFilter ref="A1:Z60"/>
   <tableColumns count="26">
     <tableColumn id="1" name="run_id"/>
     <tableColumn id="2" name="arm"/>
@@ -38765,28 +38795,28 @@
         <v>10</v>
       </c>
       <c r="E17" s="2">
-        <v>3.5348953</v>
+        <v>3.1855613000000003</v>
       </c>
       <c r="F17" s="2">
-        <v>0.4153665540195503</v>
+        <v>0.37431819262059585</v>
       </c>
       <c r="G17" s="2">
-        <v>35.348953</v>
+        <v>31.855613</v>
       </c>
       <c r="H17" s="2">
-        <v>2.46001</v>
+        <v>1.853942</v>
       </c>
       <c r="I17" s="2">
-        <v>3.517073</v>
+        <v>3.391539</v>
       </c>
       <c r="J17" s="2">
-        <v>5.325631</v>
+        <v>4.235551</v>
       </c>
       <c r="K17" s="2">
-        <v>2.8656209999999995</v>
+        <v>2.381609</v>
       </c>
       <c r="L17" s="2">
-        <v>3.517073</v>
+        <v>3.391539</v>
       </c>
       <c r="M17" s="2">
         <v>0.0</v>
@@ -38795,16 +38825,16 @@
         <v>22.31105</v>
       </c>
       <c r="O17" s="3">
-        <v>29.149991666666665</v>
+        <v>28.1522</v>
       </c>
       <c r="P17" s="3">
-        <v>38.03945</v>
+        <v>45.2761</v>
       </c>
       <c r="Q17" s="1">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="R17" s="1">
-        <v>264</v>
+        <v>232</v>
       </c>
       <c r="S17" s="1">
         <v>0</v>
@@ -38819,7 +38849,7 @@
         <v>2</v>
       </c>
       <c r="W17" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -38828,10 +38858,10 @@
         <v>0</v>
       </c>
       <c r="Z17" s="3">
-        <v>407.917</v>
+        <v>361.895</v>
       </c>
       <c r="AA17" s="3">
-        <v>565.816</v>
+        <v>549.771</v>
       </c>
     </row>
     <row r="18">
@@ -48527,12 +48557,15 @@
         <v>565816</v>
       </c>
       <c r="X133" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y133" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B134" t="s">
         <v>71</v>
@@ -48544,13 +48577,13 @@
         <v>6</v>
       </c>
       <c r="E134" t="s">
-        <v>704</v>
+        <v>110</v>
       </c>
       <c r="F134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G134" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H134" t="b">
         <v>0</v>
@@ -48558,16 +48591,52 @@
       <c r="I134" s="4">
         <v>46315.16237268518</v>
       </c>
+      <c r="J134" s="4">
+        <v>46315.19494212963</v>
+      </c>
+      <c r="K134" s="3">
+        <v>45.2761</v>
+      </c>
+      <c r="L134" s="2">
+        <v>3.470196</v>
+      </c>
+      <c r="M134" s="2">
+        <v>3.470196</v>
+      </c>
+      <c r="N134" s="2">
+        <v>0</v>
+      </c>
+      <c r="O134" s="1">
+        <v>189</v>
+      </c>
+      <c r="P134" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q134" s="1">
+        <v>0</v>
+      </c>
+      <c r="R134" s="1">
+        <v>378.0</v>
+      </c>
+      <c r="S134" s="1">
+        <v>245532.0</v>
+      </c>
+      <c r="T134" s="1">
+        <v>50940524.0</v>
+      </c>
+      <c r="U134" s="1">
+        <v>477690.0</v>
+      </c>
+      <c r="V134" s="1">
+        <v>483111</v>
+      </c>
       <c r="X134" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y134" t="s">
-        <v>705</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B135" t="s">
         <v>71</v>
@@ -48633,7 +48702,10 @@
         <v>476714</v>
       </c>
       <c r="X135" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y135" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="136">
@@ -48650,13 +48722,13 @@
         <v>7</v>
       </c>
       <c r="E136" t="s">
-        <v>704</v>
+        <v>110</v>
       </c>
       <c r="F136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G136" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H136" t="b">
         <v>0</v>
@@ -48664,11 +48736,47 @@
       <c r="I136" s="4">
         <v>46315.166493055556</v>
       </c>
+      <c r="J136" s="4">
+        <v>46315.18445601852</v>
+      </c>
+      <c r="K136" s="3">
+        <v>24.268766666666668</v>
+      </c>
+      <c r="L136" s="2">
+        <v>1.853942</v>
+      </c>
+      <c r="M136" s="2">
+        <v>1.853942</v>
+      </c>
+      <c r="N136" s="2">
+        <v>0</v>
+      </c>
+      <c r="O136" s="1">
+        <v>130</v>
+      </c>
+      <c r="P136" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q136" s="1">
+        <v>0</v>
+      </c>
+      <c r="R136" s="1">
+        <v>222.0</v>
+      </c>
+      <c r="S136" s="1">
+        <v>176469.0</v>
+      </c>
+      <c r="T136" s="1">
+        <v>23415527.0</v>
+      </c>
+      <c r="U136" s="1">
+        <v>356474.0</v>
+      </c>
+      <c r="V136" s="1">
+        <v>361895</v>
+      </c>
       <c r="X136" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y136" t="s">
-        <v>705</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -51124,11 +51232,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="54" customWidth="1"/>
+    <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
@@ -51516,43 +51624,43 @@
         <v>62</v>
       </c>
       <c r="C5" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="2">
-        <v>14.435009</v>
+        <v>13.662117</v>
       </c>
       <c r="F5" s="2">
-        <v>0.6957551475526167</v>
+        <v>0.6585024109937245</v>
       </c>
       <c r="G5" s="2">
-        <v>28.870018</v>
+        <v>40.986351</v>
       </c>
       <c r="H5" s="2">
         <v>8.11915</v>
       </c>
       <c r="I5" s="2">
-        <v>9.027269</v>
+        <v>10.375434</v>
       </c>
       <c r="J5" s="2">
-        <v>11.723599</v>
+        <v>12.116333</v>
       </c>
       <c r="K5" s="2">
-        <v>3.6044490000000007</v>
+        <v>3.9971829999999997</v>
       </c>
       <c r="L5" s="2">
-        <v>9.027269</v>
+        <v>10.375434</v>
       </c>
       <c r="M5" s="2">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="N5" s="3">
         <v>37.165499999999994</v>
       </c>
       <c r="O5" s="3">
-        <v>39.51316666666666</v>
+        <v>42.74603333333333</v>
       </c>
       <c r="P5" s="3">
         <v>200.98263333333335</v>
@@ -51688,25 +51796,25 @@
         <v>68</v>
       </c>
       <c r="C7" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" s="2">
-        <v>7.493670999999999</v>
+        <v>7.28428675</v>
       </c>
       <c r="F7" s="2">
-        <v>0.3611885640193064</v>
+        <v>0.3510964213851076</v>
       </c>
       <c r="G7" s="2">
-        <v>22.481012999999997</v>
+        <v>29.137147</v>
       </c>
       <c r="H7" s="2">
         <v>5.548321</v>
       </c>
       <c r="I7" s="2">
-        <v>8.398512</v>
+        <v>7.527323</v>
       </c>
       <c r="J7" s="2">
         <v>8.53418</v>
@@ -51715,34 +51823,34 @@
         <v>2.9858589999999996</v>
       </c>
       <c r="L7" s="2">
-        <v>8.398512</v>
+        <v>7.527323</v>
       </c>
       <c r="M7" s="2">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="N7" s="3">
-        <v>55.412016666666666</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="O7" s="3">
-        <v>59.42836666666667</v>
+        <v>57.42019166666667</v>
       </c>
       <c r="P7" s="3">
         <v>60.036500000000004</v>
       </c>
       <c r="Q7" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="R7" s="1">
         <v>32</v>
       </c>
       <c r="S7" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="1">
         <v>7</v>
       </c>
       <c r="U7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V7" s="1">
         <v>3</v>
@@ -51757,7 +51865,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="3">
-        <v>48.307</v>
+        <v>44.805</v>
       </c>
       <c r="AA7" s="3">
         <v>81.975</v>
@@ -51766,7 +51874,7 @@
         <v>299.031</v>
       </c>
       <c r="AC7" s="3">
-        <v>427.464</v>
+        <v>506.67</v>
       </c>
     </row>
     <row r="8">
@@ -52022,6 +52130,184 @@
       </c>
       <c r="AA10" s="3">
         <v>965.009</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.33877027230093076</v>
+      </c>
+      <c r="G11" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="H11" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="I11" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="J11" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="L11" s="2">
+        <v>2.251192</v>
+      </c>
+      <c r="M11" s="2">
+        <v>4.777361</v>
+      </c>
+      <c r="N11" s="3">
+        <v>47.0307</v>
+      </c>
+      <c r="O11" s="3">
+        <v>47.0307</v>
+      </c>
+      <c r="P11" s="3">
+        <v>47.0307</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>14</v>
+      </c>
+      <c r="R11" s="1">
+        <v>14</v>
+      </c>
+      <c r="S11" s="1">
+        <v>6</v>
+      </c>
+      <c r="T11" s="1">
+        <v>6</v>
+      </c>
+      <c r="U11" s="1">
+        <v>1</v>
+      </c>
+      <c r="V11" s="1">
+        <v>1</v>
+      </c>
+      <c r="W11" s="1">
+        <v>0</v>
+      </c>
+      <c r="X11" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="3">
+        <v>111.026</v>
+      </c>
+      <c r="AA11" s="3">
+        <v>111.026</v>
+      </c>
+      <c r="AB11" s="3">
+        <v>186.027</v>
+      </c>
+      <c r="AC11" s="3">
+        <v>186.027</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.4981516992055639</v>
+      </c>
+      <c r="G12" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="H12" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="I12" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="J12" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="L12" s="2">
+        <v>8.729592</v>
+      </c>
+      <c r="M12" s="2">
+        <v>1.605688</v>
+      </c>
+      <c r="N12" s="3">
+        <v>41.971066666666665</v>
+      </c>
+      <c r="O12" s="3">
+        <v>41.971066666666665</v>
+      </c>
+      <c r="P12" s="3">
+        <v>41.971066666666665</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>99</v>
+      </c>
+      <c r="R12" s="1">
+        <v>99</v>
+      </c>
+      <c r="S12" s="1">
+        <v>2</v>
+      </c>
+      <c r="T12" s="1">
+        <v>2</v>
+      </c>
+      <c r="U12" s="1">
+        <v>1</v>
+      </c>
+      <c r="V12" s="1">
+        <v>1</v>
+      </c>
+      <c r="W12" s="1">
+        <v>0</v>
+      </c>
+      <c r="X12" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="3">
+        <v>294.098</v>
+      </c>
+      <c r="AA12" s="3">
+        <v>294.098</v>
+      </c>
+      <c r="AB12" s="3">
+        <v>126.892</v>
+      </c>
+      <c r="AC12" s="3">
+        <v>126.892</v>
       </c>
     </row>
   </sheetData>
@@ -52033,12 +52319,12 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z52"/>
+  <dimension ref="A1:Z60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="7" customWidth="1"/>
-    <col min="3" max="3" width="54" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
@@ -53893,31 +54179,31 @@
         <v>1</v>
       </c>
       <c r="G25" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" t="b">
         <v>0</v>
       </c>
       <c r="I25" s="4">
-        <v>46314.158472222225</v>
+        <v>46315.19474537037</v>
       </c>
       <c r="J25" s="4">
-        <v>46314.19175925926</v>
+        <v>46315.23090277778</v>
       </c>
       <c r="K25" s="3">
-        <v>37.165499999999994</v>
+        <v>45.978899999999996</v>
       </c>
       <c r="L25" s="2">
-        <v>9.027269</v>
+        <v>12.116333</v>
       </c>
       <c r="M25" s="2">
-        <v>9.027269</v>
+        <v>12.116332</v>
       </c>
       <c r="N25" s="2">
         <v>0</v>
       </c>
       <c r="O25" s="1">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P25" s="1">
         <v>5</v>
@@ -53926,22 +54212,22 @@
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>862.0</v>
+        <v>854.0</v>
       </c>
       <c r="S25" s="1">
-        <v>916295.0</v>
+        <v>831298.0</v>
       </c>
       <c r="T25" s="1">
-        <v>70004365.0</v>
+        <v>82990864.0</v>
       </c>
       <c r="U25" s="1">
-        <v>1517336.0</v>
+        <v>1403045.0</v>
       </c>
       <c r="V25" s="1">
-        <v>293858</v>
+        <v>405401</v>
       </c>
       <c r="W25" s="1">
-        <v>362172</v>
+        <v>371552</v>
       </c>
       <c r="X25" t="b">
         <v>1</v>
@@ -53958,13 +54244,13 @@
         <v>62</v>
       </c>
       <c r="D26" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="1">
         <v>2</v>
@@ -53973,58 +54259,52 @@
         <v>0</v>
       </c>
       <c r="I26" s="4">
-        <v>46314.15987268519</v>
+        <v>46314.158472222225</v>
       </c>
       <c r="J26" s="4">
-        <v>46314.19658564815</v>
+        <v>46314.19175925926</v>
       </c>
       <c r="K26" s="3">
-        <v>47.48878333333334</v>
+        <v>37.165499999999994</v>
       </c>
       <c r="L26" s="2">
-        <v>5.239723</v>
+        <v>9.027269</v>
       </c>
       <c r="M26" s="2">
-        <v>5.239722</v>
+        <v>9.027269</v>
       </c>
       <c r="N26" s="2">
         <v>0</v>
       </c>
       <c r="O26" s="1">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="P26" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q26" s="1">
         <v>0</v>
       </c>
       <c r="R26" s="1">
-        <v>718.0</v>
+        <v>862.0</v>
       </c>
       <c r="S26" s="1">
-        <v>792807.0</v>
+        <v>916295.0</v>
       </c>
       <c r="T26" s="1">
-        <v>61846940.0</v>
+        <v>70004365.0</v>
       </c>
       <c r="U26" s="1">
-        <v>1339689.0</v>
+        <v>1517336.0</v>
       </c>
       <c r="V26" s="1">
-        <v>289296</v>
+        <v>293858</v>
       </c>
       <c r="W26" s="1">
-        <v>386280</v>
+        <v>362172</v>
       </c>
       <c r="X26" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y26" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z26" t="s">
-        <v>748</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -54047,55 +54327,55 @@
         <v>0</v>
       </c>
       <c r="G27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H27" t="b">
         <v>0</v>
       </c>
       <c r="I27" s="4">
-        <v>46313.890914351854</v>
+        <v>46314.15987268519</v>
       </c>
       <c r="J27" s="4">
-        <v>46313.904699074075</v>
+        <v>46314.19658564815</v>
       </c>
       <c r="K27" s="3">
-        <v>19.798949999999998</v>
+        <v>47.48878333333334</v>
       </c>
       <c r="L27" s="2">
-        <v>4.110965</v>
+        <v>5.239723</v>
       </c>
       <c r="M27" s="2">
-        <v>4.110965</v>
+        <v>5.239722</v>
       </c>
       <c r="N27" s="2">
         <v>0</v>
       </c>
       <c r="O27" s="1">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="P27" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q27" s="1">
         <v>0</v>
       </c>
       <c r="R27" s="1">
-        <v>242.0</v>
+        <v>718.0</v>
       </c>
       <c r="S27" s="1">
-        <v>222561.0</v>
+        <v>792807.0</v>
       </c>
       <c r="T27" s="1">
-        <v>17740423.0</v>
+        <v>61846940.0</v>
       </c>
       <c r="U27" s="1">
-        <v>428109.0</v>
+        <v>1339689.0</v>
       </c>
       <c r="V27" s="1">
-        <v>273440</v>
+        <v>289296</v>
       </c>
       <c r="W27" s="1">
-        <v>164825</v>
+        <v>386280</v>
       </c>
       <c r="X27" t="b">
         <v>0</v>
@@ -54104,7 +54384,7 @@
         <v>432</v>
       </c>
       <c r="Z27" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
     </row>
     <row r="28">
@@ -54121,64 +54401,70 @@
         <v>2</v>
       </c>
       <c r="E28" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
       </c>
       <c r="G28" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" s="4">
-        <v>46314.52525462963</v>
+        <v>46313.890914351854</v>
       </c>
       <c r="J28" s="4">
-        <v>46314.68326388889</v>
+        <v>46313.904699074075</v>
       </c>
       <c r="K28" s="3">
-        <v>200.98263333333335</v>
+        <v>19.798949999999998</v>
       </c>
       <c r="L28" s="2">
-        <v>11.723599</v>
+        <v>4.110965</v>
       </c>
       <c r="M28" s="2">
-        <v>11.723599</v>
+        <v>4.110965</v>
       </c>
       <c r="N28" s="2">
         <v>0</v>
       </c>
       <c r="O28" s="1">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="P28" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q28" s="1">
         <v>0</v>
       </c>
       <c r="R28" s="1">
-        <v>1574.0</v>
+        <v>242.0</v>
       </c>
       <c r="S28" s="1">
-        <v>1447397.0</v>
+        <v>222561.0</v>
       </c>
       <c r="T28" s="1">
-        <v>141502391.0</v>
+        <v>17740423.0</v>
       </c>
       <c r="U28" s="1">
-        <v>3602058.0</v>
+        <v>428109.0</v>
       </c>
       <c r="V28" s="1">
-        <v>458412</v>
+        <v>273440</v>
       </c>
       <c r="W28" s="1">
-        <v>477389</v>
+        <v>164825</v>
       </c>
       <c r="X28" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>746</v>
       </c>
     </row>
     <row r="29">
@@ -54192,64 +54478,64 @@
         <v>62</v>
       </c>
       <c r="D29" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" t="s">
         <v>110</v>
       </c>
       <c r="F29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" s="4">
-        <v>46314.29790509259</v>
+        <v>46314.52525462963</v>
       </c>
       <c r="J29" s="4">
-        <v>46314.32916666667</v>
+        <v>46314.68326388889</v>
       </c>
       <c r="K29" s="3">
-        <v>39.51316666666666</v>
+        <v>200.98263333333335</v>
       </c>
       <c r="L29" s="2">
-        <v>8.11915</v>
+        <v>11.723599</v>
       </c>
       <c r="M29" s="2">
-        <v>8.11915</v>
+        <v>11.723599</v>
       </c>
       <c r="N29" s="2">
         <v>0</v>
       </c>
       <c r="O29" s="1">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="P29" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Q29" s="1">
         <v>0</v>
       </c>
       <c r="R29" s="1">
-        <v>666.0</v>
+        <v>1574.0</v>
       </c>
       <c r="S29" s="1">
-        <v>710400.0</v>
+        <v>1447397.0</v>
       </c>
       <c r="T29" s="1">
-        <v>55968395.0</v>
+        <v>141502391.0</v>
       </c>
       <c r="U29" s="1">
-        <v>1169834.0</v>
+        <v>3602058.0</v>
       </c>
       <c r="V29" s="1">
-        <v>312594</v>
+        <v>458412</v>
       </c>
       <c r="W29" s="1">
-        <v>322948</v>
+        <v>477389</v>
       </c>
       <c r="X29" t="b">
         <v>1</v>
@@ -54260,158 +54546,113 @@
         <v>776</v>
       </c>
       <c r="B30" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D30" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>431</v>
+        <v>777</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
       </c>
       <c r="G30" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H30" t="b">
         <v>0</v>
       </c>
       <c r="I30" s="4">
-        <v>46314.15864583333</v>
-      </c>
-      <c r="J30" s="4">
-        <v>46314.19634259259</v>
-      </c>
-      <c r="K30" s="3">
-        <v>48.41158333333333</v>
-      </c>
-      <c r="L30" s="2">
-        <v>8.756337</v>
-      </c>
-      <c r="M30" s="2">
-        <v>8.756337</v>
-      </c>
-      <c r="N30" s="2">
-        <v>0</v>
-      </c>
-      <c r="O30" s="1">
-        <v>146</v>
-      </c>
-      <c r="P30" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="1">
-        <v>0</v>
-      </c>
-      <c r="R30" s="1">
-        <v>282.0</v>
-      </c>
-      <c r="S30" s="1">
-        <v>279123.0</v>
-      </c>
-      <c r="T30" s="1">
-        <v>40577429.0</v>
-      </c>
-      <c r="U30" s="1">
-        <v>476700.0</v>
-      </c>
-      <c r="V30" s="1">
-        <v>476702</v>
+        <v>46315.22869212963</v>
       </c>
       <c r="X30" t="b">
         <v>0</v>
       </c>
       <c r="Y30" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z30" t="s">
-        <v>748</v>
+        <v>778</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D31" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H31" t="b">
         <v>0</v>
       </c>
       <c r="I31" s="4">
-        <v>46313.86145833333</v>
+        <v>46314.29790509259</v>
       </c>
       <c r="J31" s="4">
-        <v>46313.90385416667</v>
+        <v>46314.32916666667</v>
       </c>
       <c r="K31" s="3">
-        <v>54.91406666666667</v>
+        <v>39.51316666666666</v>
       </c>
       <c r="L31" s="2">
-        <v>10.22348</v>
+        <v>8.11915</v>
       </c>
       <c r="M31" s="2">
-        <v>10.22348</v>
+        <v>8.11915</v>
       </c>
       <c r="N31" s="2">
         <v>0</v>
       </c>
       <c r="O31" s="1">
-        <v>165</v>
+        <v>16</v>
       </c>
       <c r="P31" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
-        <v>320.0</v>
+        <v>666.0</v>
       </c>
       <c r="S31" s="1">
-        <v>299935.0</v>
+        <v>710400.0</v>
       </c>
       <c r="T31" s="1">
-        <v>51508661.0</v>
+        <v>55968395.0</v>
       </c>
       <c r="U31" s="1">
-        <v>518156.0</v>
+        <v>1169834.0</v>
       </c>
       <c r="V31" s="1">
-        <v>523577</v>
+        <v>312594</v>
+      </c>
+      <c r="W31" s="1">
+        <v>322948</v>
       </c>
       <c r="X31" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y31" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z31" t="s">
-        <v>753</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="B32" t="s">
         <v>63</v>
@@ -54423,10 +54664,10 @@
         <v>1</v>
       </c>
       <c r="E32" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="1">
         <v>2</v>
@@ -54435,25 +54676,25 @@
         <v>0</v>
       </c>
       <c r="I32" s="4">
-        <v>46314.57332175926</v>
+        <v>46314.15864583333</v>
       </c>
       <c r="J32" s="4">
-        <v>46314.61576388889</v>
+        <v>46314.19634259259</v>
       </c>
       <c r="K32" s="3">
-        <v>50.72746666666667</v>
+        <v>48.41158333333333</v>
       </c>
       <c r="L32" s="2">
-        <v>11.371427</v>
+        <v>8.756337</v>
       </c>
       <c r="M32" s="2">
-        <v>11.371427</v>
+        <v>8.756337</v>
       </c>
       <c r="N32" s="2">
         <v>0</v>
       </c>
       <c r="O32" s="1">
-        <v>178</v>
+        <v>146</v>
       </c>
       <c r="P32" s="1">
         <v>0</v>
@@ -54462,27 +54703,33 @@
         <v>0</v>
       </c>
       <c r="R32" s="1">
-        <v>352.0</v>
+        <v>282.0</v>
       </c>
       <c r="S32" s="1">
-        <v>323735.0</v>
+        <v>279123.0</v>
       </c>
       <c r="T32" s="1">
-        <v>58971088.0</v>
+        <v>40577429.0</v>
       </c>
       <c r="U32" s="1">
-        <v>559066.0</v>
+        <v>476700.0</v>
       </c>
       <c r="V32" s="1">
-        <v>559068</v>
+        <v>476702</v>
       </c>
       <c r="X32" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>748</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="B33" t="s">
         <v>63</v>
@@ -54491,40 +54738,40 @@
         <v>64</v>
       </c>
       <c r="D33" s="1">
+        <v>1</v>
+      </c>
+      <c r="E33" t="s">
+        <v>431</v>
+      </c>
+      <c r="F33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1">
         <v>2</v>
       </c>
-      <c r="E33" t="s">
-        <v>110</v>
-      </c>
-      <c r="F33" t="b">
-        <v>1</v>
-      </c>
-      <c r="G33" s="1">
-        <v>1</v>
-      </c>
       <c r="H33" t="b">
         <v>0</v>
       </c>
       <c r="I33" s="4">
-        <v>46314.160046296296</v>
+        <v>46313.86145833333</v>
       </c>
       <c r="J33" s="4">
-        <v>46314.19709490741</v>
+        <v>46313.90385416667</v>
       </c>
       <c r="K33" s="3">
-        <v>48.04756666666666</v>
+        <v>54.91406666666667</v>
       </c>
       <c r="L33" s="2">
-        <v>9.165487</v>
+        <v>10.22348</v>
       </c>
       <c r="M33" s="2">
-        <v>9.165487</v>
+        <v>10.22348</v>
       </c>
       <c r="N33" s="2">
         <v>0</v>
       </c>
       <c r="O33" s="1">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="P33" s="1">
         <v>0</v>
@@ -54533,27 +54780,33 @@
         <v>0</v>
       </c>
       <c r="R33" s="1">
-        <v>294.0</v>
+        <v>320.0</v>
       </c>
       <c r="S33" s="1">
-        <v>289718.0</v>
+        <v>299935.0</v>
       </c>
       <c r="T33" s="1">
-        <v>42949072.0</v>
+        <v>51508661.0</v>
       </c>
       <c r="U33" s="1">
-        <v>493203.0</v>
+        <v>518156.0</v>
       </c>
       <c r="V33" s="1">
-        <v>498624</v>
+        <v>523577</v>
       </c>
       <c r="X33" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>753</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="B34" t="s">
         <v>63</v>
@@ -54562,40 +54815,40 @@
         <v>64</v>
       </c>
       <c r="D34" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E34" t="s">
         <v>110</v>
       </c>
       <c r="F34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I34" s="4">
-        <v>46314.32548611111</v>
+        <v>46314.57332175926</v>
       </c>
       <c r="J34" s="4">
-        <v>46314.41706018519</v>
+        <v>46314.61576388889</v>
       </c>
       <c r="K34" s="3">
-        <v>104.91581666666666</v>
+        <v>50.72746666666667</v>
       </c>
       <c r="L34" s="2">
-        <v>21.168002</v>
+        <v>11.371427</v>
       </c>
       <c r="M34" s="2">
-        <v>21.168002</v>
+        <v>11.371427</v>
       </c>
       <c r="N34" s="2">
         <v>0</v>
       </c>
       <c r="O34" s="1">
-        <v>98</v>
+        <v>178</v>
       </c>
       <c r="P34" s="1">
         <v>0</v>
@@ -54604,19 +54857,19 @@
         <v>0</v>
       </c>
       <c r="R34" s="1">
-        <v>582.0</v>
+        <v>352.0</v>
       </c>
       <c r="S34" s="1">
-        <v>498236.0</v>
+        <v>323735.0</v>
       </c>
       <c r="T34" s="1">
-        <v>131478461.0</v>
+        <v>58971088.0</v>
       </c>
       <c r="U34" s="1">
-        <v>759158.0</v>
+        <v>559066.0</v>
       </c>
       <c r="V34" s="1">
-        <v>764579</v>
+        <v>559068</v>
       </c>
       <c r="X34" t="b">
         <v>1</v>
@@ -54624,153 +54877,141 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D35" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H35" t="b">
         <v>0</v>
       </c>
       <c r="I35" s="4">
-        <v>46313.86164351852</v>
+        <v>46314.160046296296</v>
       </c>
       <c r="J35" s="4">
-        <v>46313.90555555555</v>
+        <v>46314.19709490741</v>
       </c>
       <c r="K35" s="3">
-        <v>51.99661666666667</v>
+        <v>48.04756666666666</v>
       </c>
       <c r="L35" s="2">
-        <v>7.706352</v>
+        <v>9.165487</v>
       </c>
       <c r="M35" s="2">
-        <v>7.706352</v>
+        <v>9.165487</v>
       </c>
       <c r="N35" s="2">
         <v>0</v>
       </c>
       <c r="O35" s="1">
-        <v>28</v>
+        <v>150</v>
       </c>
       <c r="P35" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Q35" s="1">
         <v>0</v>
       </c>
       <c r="R35" s="1">
-        <v>924.0</v>
+        <v>294.0</v>
       </c>
       <c r="S35" s="1">
-        <v>779272.0</v>
+        <v>289718.0</v>
       </c>
       <c r="T35" s="1">
-        <v>48456621.0</v>
+        <v>42949072.0</v>
       </c>
       <c r="U35" s="1">
-        <v>1705620.0</v>
+        <v>493203.0</v>
       </c>
       <c r="V35" s="1">
-        <v>85496</v>
-      </c>
-      <c r="W35" s="1">
-        <v>257260</v>
+        <v>498624</v>
       </c>
       <c r="X35" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y35" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z35" t="s">
-        <v>782</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D36" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E36" t="s">
         <v>110</v>
       </c>
       <c r="F36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" s="4">
-        <v>46314.584178240744</v>
+        <v>46314.32548611111</v>
       </c>
       <c r="J36" s="4">
-        <v>46314.63313657408</v>
+        <v>46314.41706018519</v>
       </c>
       <c r="K36" s="3">
-        <v>60.036500000000004</v>
+        <v>104.91581666666666</v>
       </c>
       <c r="L36" s="2">
-        <v>5.548321</v>
+        <v>21.168002</v>
       </c>
       <c r="M36" s="2">
-        <v>5.548322</v>
+        <v>21.168002</v>
       </c>
       <c r="N36" s="2">
         <v>0</v>
       </c>
       <c r="O36" s="1">
-        <v>16</v>
+        <v>98</v>
       </c>
       <c r="P36" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q36" s="1">
         <v>0</v>
       </c>
       <c r="R36" s="1">
-        <v>520.0</v>
+        <v>582.0</v>
       </c>
       <c r="S36" s="1">
-        <v>539478.0</v>
+        <v>498236.0</v>
       </c>
       <c r="T36" s="1">
-        <v>36078318.0</v>
+        <v>131478461.0</v>
       </c>
       <c r="U36" s="1">
-        <v>948571.0</v>
+        <v>759158.0</v>
       </c>
       <c r="V36" s="1">
-        <v>48307</v>
-      </c>
-      <c r="W36" s="1">
-        <v>380955</v>
+        <v>764579</v>
       </c>
       <c r="X36" t="b">
         <v>1</v>
@@ -54778,7 +55019,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="B37" t="s">
         <v>67</v>
@@ -54796,55 +55037,55 @@
         <v>0</v>
       </c>
       <c r="G37" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H37" t="b">
         <v>0</v>
       </c>
       <c r="I37" s="4">
-        <v>46314.15881944444</v>
+        <v>46313.86164351852</v>
       </c>
       <c r="J37" s="4">
-        <v>46314.19364583334</v>
+        <v>46313.90555555555</v>
       </c>
       <c r="K37" s="3">
-        <v>44.1155</v>
+        <v>51.99661666666667</v>
       </c>
       <c r="L37" s="2">
-        <v>3.875124</v>
+        <v>7.706352</v>
       </c>
       <c r="M37" s="2">
-        <v>3.875124</v>
+        <v>7.706352</v>
       </c>
       <c r="N37" s="2">
         <v>0</v>
       </c>
       <c r="O37" s="1">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="P37" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="Q37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
-        <v>540.0</v>
+        <v>924.0</v>
       </c>
       <c r="S37" s="1">
-        <v>529894.0</v>
+        <v>779272.0</v>
       </c>
       <c r="T37" s="1">
-        <v>35974215.0</v>
+        <v>48456621.0</v>
       </c>
       <c r="U37" s="1">
-        <v>997521.0</v>
+        <v>1705620.0</v>
       </c>
       <c r="V37" s="1">
-        <v>47980</v>
+        <v>85496</v>
       </c>
       <c r="W37" s="1">
-        <v>293478</v>
+        <v>257260</v>
       </c>
       <c r="X37" t="b">
         <v>0</v>
@@ -54853,12 +55094,12 @@
         <v>432</v>
       </c>
       <c r="Z37" t="s">
-        <v>748</v>
+        <v>786</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="B38" t="s">
         <v>67</v>
@@ -54867,7 +55108,7 @@
         <v>68</v>
       </c>
       <c r="D38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
         <v>110</v>
@@ -54876,55 +55117,55 @@
         <v>1</v>
       </c>
       <c r="G38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H38" t="b">
         <v>0</v>
       </c>
       <c r="I38" s="4">
-        <v>46314.210381944446</v>
+        <v>46315.19493055555</v>
       </c>
       <c r="J38" s="4">
-        <v>46314.25950231482</v>
+        <v>46315.23050925926</v>
       </c>
       <c r="K38" s="3">
-        <v>59.42836666666667</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="L38" s="2">
-        <v>8.398512</v>
+        <v>6.656134</v>
       </c>
       <c r="M38" s="2">
-        <v>8.398512</v>
+        <v>6.656134</v>
       </c>
       <c r="N38" s="2">
         <v>0</v>
       </c>
       <c r="O38" s="1">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="P38" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
-        <v>618.0</v>
+        <v>460.0</v>
       </c>
       <c r="S38" s="1">
-        <v>621706.0</v>
+        <v>509481.0</v>
       </c>
       <c r="T38" s="1">
-        <v>54903298.0</v>
+        <v>44845086.0</v>
       </c>
       <c r="U38" s="1">
-        <v>1155513.0</v>
+        <v>861558.0</v>
       </c>
       <c r="V38" s="1">
-        <v>64109</v>
+        <v>44805</v>
       </c>
       <c r="W38" s="1">
-        <v>427464</v>
+        <v>506670</v>
       </c>
       <c r="X38" t="b">
         <v>1</v>
@@ -54932,7 +55173,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="B39" t="s">
         <v>67</v>
@@ -54941,7 +55182,7 @@
         <v>68</v>
       </c>
       <c r="D39" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E39" t="s">
         <v>110</v>
@@ -54950,55 +55191,55 @@
         <v>1</v>
       </c>
       <c r="G39" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H39" t="b">
         <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>46314.32938657407</v>
+        <v>46314.584178240744</v>
       </c>
       <c r="J39" s="4">
-        <v>46314.379849537036</v>
+        <v>46314.63313657408</v>
       </c>
       <c r="K39" s="3">
-        <v>55.412016666666666</v>
+        <v>60.036500000000004</v>
       </c>
       <c r="L39" s="2">
-        <v>8.53418</v>
+        <v>5.548321</v>
       </c>
       <c r="M39" s="2">
-        <v>8.53418</v>
+        <v>5.548322</v>
       </c>
       <c r="N39" s="2">
         <v>0</v>
       </c>
       <c r="O39" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="P39" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
-        <v>834.0</v>
+        <v>520.0</v>
       </c>
       <c r="S39" s="1">
-        <v>839688.0</v>
+        <v>539478.0</v>
       </c>
       <c r="T39" s="1">
-        <v>54499916.0</v>
+        <v>36078318.0</v>
       </c>
       <c r="U39" s="1">
-        <v>1684516.0</v>
+        <v>948571.0</v>
       </c>
       <c r="V39" s="1">
-        <v>81975</v>
+        <v>48307</v>
       </c>
       <c r="W39" s="1">
-        <v>299031</v>
+        <v>380955</v>
       </c>
       <c r="X39" t="b">
         <v>1</v>
@@ -55006,13 +55247,13 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D40" s="1">
         <v>1</v>
@@ -55024,55 +55265,55 @@
         <v>0</v>
       </c>
       <c r="G40" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40" t="b">
         <v>0</v>
       </c>
       <c r="I40" s="4">
-        <v>46314.15899305556</v>
+        <v>46314.15881944444</v>
       </c>
       <c r="J40" s="4">
-        <v>46314.193460648145</v>
+        <v>46314.19364583334</v>
       </c>
       <c r="K40" s="3">
-        <v>49.385549999999995</v>
+        <v>44.1155</v>
       </c>
       <c r="L40" s="2">
-        <v>10.350417</v>
+        <v>3.875124</v>
       </c>
       <c r="M40" s="2">
-        <v>10.350418</v>
+        <v>3.875124</v>
       </c>
       <c r="N40" s="2">
         <v>0</v>
       </c>
       <c r="O40" s="1">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="P40" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q40" s="1">
         <v>0</v>
       </c>
       <c r="R40" s="1">
-        <v>1084.0</v>
+        <v>540.0</v>
       </c>
       <c r="S40" s="1">
-        <v>986438.0</v>
+        <v>529894.0</v>
       </c>
       <c r="T40" s="1">
-        <v>88431683.0</v>
+        <v>35974215.0</v>
       </c>
       <c r="U40" s="1">
-        <v>1905956.0</v>
+        <v>997521.0</v>
       </c>
       <c r="V40" s="1">
-        <v>236869</v>
+        <v>47980</v>
       </c>
       <c r="W40" s="1">
-        <v>376179</v>
+        <v>293478</v>
       </c>
       <c r="X40" t="b">
         <v>0</v>
@@ -55081,27 +55322,27 @@
         <v>432</v>
       </c>
       <c r="Z40" t="s">
-        <v>788</v>
+        <v>748</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C41" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D41" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" s="1">
         <v>2</v>
@@ -55110,25 +55351,25 @@
         <v>0</v>
       </c>
       <c r="I41" s="4">
-        <v>46313.862280092595</v>
+        <v>46314.210381944446</v>
       </c>
       <c r="J41" s="4">
-        <v>46313.90387731481</v>
+        <v>46314.25950231482</v>
       </c>
       <c r="K41" s="3">
-        <v>54.19301666666667</v>
+        <v>59.42836666666667</v>
       </c>
       <c r="L41" s="2">
-        <v>11.580787</v>
+        <v>8.398512</v>
       </c>
       <c r="M41" s="2">
-        <v>11.580788</v>
+        <v>8.398512</v>
       </c>
       <c r="N41" s="2">
         <v>0</v>
       </c>
       <c r="O41" s="1">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="P41" s="1">
         <v>4</v>
@@ -55137,119 +55378,74 @@
         <v>0</v>
       </c>
       <c r="R41" s="1">
-        <v>576.0</v>
+        <v>618.0</v>
       </c>
       <c r="S41" s="1">
-        <v>486536.0</v>
+        <v>621706.0</v>
       </c>
       <c r="T41" s="1">
-        <v>43600123.0</v>
+        <v>54903298.0</v>
       </c>
       <c r="U41" s="1">
-        <v>1090895.0</v>
+        <v>1155513.0</v>
       </c>
       <c r="V41" s="1">
-        <v>157439</v>
+        <v>64109</v>
       </c>
       <c r="W41" s="1">
-        <v>369085</v>
+        <v>427464</v>
       </c>
       <c r="X41" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y41" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z41" t="s">
-        <v>753</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C42" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" t="s">
-        <v>110</v>
+        <v>777</v>
       </c>
       <c r="F42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G42" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H42" t="b">
         <v>0</v>
       </c>
       <c r="I42" s="4">
-        <v>46314.586909722224</v>
-      </c>
-      <c r="J42" s="4">
-        <v>46314.640069444446</v>
-      </c>
-      <c r="K42" s="3">
-        <v>65.17911666666666</v>
-      </c>
-      <c r="L42" s="2">
-        <v>10.446109</v>
-      </c>
-      <c r="M42" s="2">
-        <v>10.446109</v>
-      </c>
-      <c r="N42" s="2">
-        <v>0</v>
-      </c>
-      <c r="O42" s="1">
-        <v>35</v>
-      </c>
-      <c r="P42" s="1">
-        <v>5</v>
-      </c>
-      <c r="Q42" s="1">
-        <v>0</v>
-      </c>
-      <c r="R42" s="1">
-        <v>722.0</v>
-      </c>
-      <c r="S42" s="1">
-        <v>708289.0</v>
-      </c>
-      <c r="T42" s="1">
-        <v>51642018.0</v>
-      </c>
-      <c r="U42" s="1">
-        <v>1305105.0</v>
-      </c>
-      <c r="V42" s="1">
-        <v>179932</v>
-      </c>
-      <c r="W42" s="1">
-        <v>420234</v>
+        <v>46315.230729166666</v>
       </c>
       <c r="X42" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>778</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B43" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C43" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D43" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" t="s">
         <v>110</v>
@@ -55264,49 +55460,49 @@
         <v>0</v>
       </c>
       <c r="I43" s="4">
-        <v>46314.21055555555</v>
+        <v>46314.32938657407</v>
       </c>
       <c r="J43" s="4">
-        <v>46314.25184027778</v>
+        <v>46314.379849537036</v>
       </c>
       <c r="K43" s="3">
-        <v>48.78155</v>
+        <v>55.412016666666666</v>
       </c>
       <c r="L43" s="2">
-        <v>12.718512</v>
+        <v>8.53418</v>
       </c>
       <c r="M43" s="2">
-        <v>12.718512</v>
+        <v>8.53418</v>
       </c>
       <c r="N43" s="2">
         <v>0</v>
       </c>
       <c r="O43" s="1">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="P43" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
-        <v>882.0</v>
+        <v>834.0</v>
       </c>
       <c r="S43" s="1">
-        <v>945280.0</v>
+        <v>839688.0</v>
       </c>
       <c r="T43" s="1">
-        <v>64072835.0</v>
+        <v>54499916.0</v>
       </c>
       <c r="U43" s="1">
-        <v>1711070.0</v>
+        <v>1684516.0</v>
       </c>
       <c r="V43" s="1">
-        <v>223412</v>
+        <v>81975</v>
       </c>
       <c r="W43" s="1">
-        <v>358765</v>
+        <v>299031</v>
       </c>
       <c r="X43" t="b">
         <v>1</v>
@@ -55314,7 +55510,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B44" t="s">
         <v>69</v>
@@ -55323,158 +55519,173 @@
         <v>70</v>
       </c>
       <c r="D44" s="1">
+        <v>1</v>
+      </c>
+      <c r="E44" t="s">
+        <v>431</v>
+      </c>
+      <c r="F44" t="b">
+        <v>0</v>
+      </c>
+      <c r="G44" s="1">
         <v>3</v>
       </c>
-      <c r="E44" t="s">
-        <v>110</v>
-      </c>
-      <c r="F44" t="b">
-        <v>1</v>
-      </c>
-      <c r="G44" s="1">
-        <v>2</v>
-      </c>
       <c r="H44" t="b">
         <v>0</v>
       </c>
       <c r="I44" s="4">
-        <v>46314.33002314815</v>
+        <v>46314.15899305556</v>
       </c>
       <c r="J44" s="4">
-        <v>46314.3778125</v>
+        <v>46314.193460648145</v>
       </c>
       <c r="K44" s="3">
-        <v>58.06751666666666</v>
+        <v>49.385549999999995</v>
       </c>
       <c r="L44" s="2">
-        <v>9.519687</v>
+        <v>10.350417</v>
       </c>
       <c r="M44" s="2">
-        <v>9.519686</v>
+        <v>10.350418</v>
       </c>
       <c r="N44" s="2">
         <v>0</v>
       </c>
       <c r="O44" s="1">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="P44" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
-        <v>528.0</v>
+        <v>1084.0</v>
       </c>
       <c r="S44" s="1">
-        <v>564432.0</v>
+        <v>986438.0</v>
       </c>
       <c r="T44" s="1">
-        <v>41322323.0</v>
+        <v>88431683.0</v>
       </c>
       <c r="U44" s="1">
-        <v>971256.0</v>
+        <v>1905956.0</v>
       </c>
       <c r="V44" s="1">
-        <v>132839</v>
+        <v>236869</v>
       </c>
       <c r="W44" s="1">
-        <v>445527</v>
+        <v>376179</v>
       </c>
       <c r="X44" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C45" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D45" s="1">
         <v>1</v>
       </c>
       <c r="E45" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H45" t="b">
         <v>0</v>
       </c>
       <c r="I45" s="4">
-        <v>46314.59266203704</v>
+        <v>46313.862280092595</v>
       </c>
       <c r="J45" s="4">
-        <v>46314.654490740744</v>
+        <v>46313.90387731481</v>
       </c>
       <c r="K45" s="3">
-        <v>73.2598</v>
+        <v>54.19301666666667</v>
       </c>
       <c r="L45" s="2">
-        <v>9.924175</v>
+        <v>11.580787</v>
       </c>
       <c r="M45" s="2">
-        <v>9.924175</v>
+        <v>11.580788</v>
       </c>
       <c r="N45" s="2">
         <v>0</v>
       </c>
       <c r="O45" s="1">
-        <v>293</v>
+        <v>23</v>
       </c>
       <c r="P45" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
-        <v>582.0</v>
+        <v>576.0</v>
       </c>
       <c r="S45" s="1">
-        <v>644532.0</v>
+        <v>486536.0</v>
       </c>
       <c r="T45" s="1">
-        <v>151776389.0</v>
+        <v>43600123.0</v>
       </c>
       <c r="U45" s="1">
-        <v>884968.0</v>
+        <v>1090895.0</v>
       </c>
       <c r="V45" s="1">
-        <v>884970</v>
+        <v>157439</v>
+      </c>
+      <c r="W45" s="1">
+        <v>369085</v>
       </c>
       <c r="X45" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>753</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C46" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D46" s="1">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="1">
         <v>2</v>
@@ -55483,66 +55694,63 @@
         <v>0</v>
       </c>
       <c r="I46" s="4">
-        <v>46314.159166666665</v>
+        <v>46314.586909722224</v>
       </c>
       <c r="J46" s="4">
-        <v>46314.19351851852</v>
+        <v>46314.640069444446</v>
       </c>
       <c r="K46" s="3">
-        <v>43.80995</v>
+        <v>65.17911666666666</v>
       </c>
       <c r="L46" s="2">
-        <v>1.351832</v>
+        <v>10.446109</v>
       </c>
       <c r="M46" s="2">
-        <v>1.351832</v>
+        <v>10.446109</v>
       </c>
       <c r="N46" s="2">
         <v>0</v>
       </c>
       <c r="O46" s="1">
-        <v>235</v>
+        <v>35</v>
       </c>
       <c r="P46" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
-        <v>432.0</v>
+        <v>722.0</v>
       </c>
       <c r="S46" s="1">
-        <v>538506.0</v>
+        <v>708289.0</v>
       </c>
       <c r="T46" s="1">
-        <v>92764505.0</v>
+        <v>51642018.0</v>
       </c>
       <c r="U46" s="1">
-        <v>774455.0</v>
+        <v>1305105.0</v>
       </c>
       <c r="V46" s="1">
-        <v>779876</v>
+        <v>179932</v>
+      </c>
+      <c r="W46" s="1">
+        <v>420234</v>
       </c>
       <c r="X46" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y46" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z46" t="s">
-        <v>748</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="B47" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C47" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D47" s="1">
         <v>2</v>
@@ -55551,55 +55759,58 @@
         <v>110</v>
       </c>
       <c r="F47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I47" s="4">
-        <v>46314.21072916667</v>
+        <v>46314.21055555555</v>
       </c>
       <c r="J47" s="4">
-        <v>46314.29785879629</v>
+        <v>46314.25184027778</v>
       </c>
       <c r="K47" s="3">
-        <v>99.19116666666667</v>
+        <v>48.78155</v>
       </c>
       <c r="L47" s="2">
-        <v>14.433891</v>
+        <v>12.718512</v>
       </c>
       <c r="M47" s="2">
-        <v>14.433891</v>
+        <v>12.718512</v>
       </c>
       <c r="N47" s="2">
         <v>0</v>
       </c>
       <c r="O47" s="1">
-        <v>182</v>
+        <v>51</v>
       </c>
       <c r="P47" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q47" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R47" s="1">
-        <v>944.0</v>
+        <v>882.0</v>
       </c>
       <c r="S47" s="1">
-        <v>719044.0</v>
+        <v>945280.0</v>
       </c>
       <c r="T47" s="1">
-        <v>235843525.0</v>
+        <v>64072835.0</v>
       </c>
       <c r="U47" s="1">
-        <v>1151474.0</v>
+        <v>1711070.0</v>
       </c>
       <c r="V47" s="1">
-        <v>963737</v>
+        <v>223412</v>
+      </c>
+      <c r="W47" s="1">
+        <v>358765</v>
       </c>
       <c r="X47" t="b">
         <v>1</v>
@@ -55607,13 +55818,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C48" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D48" s="1">
         <v>3</v>
@@ -55622,55 +55833,58 @@
         <v>110</v>
       </c>
       <c r="F48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I48" s="4">
-        <v>46314.354363425926</v>
+        <v>46314.33002314815</v>
       </c>
       <c r="J48" s="4">
-        <v>46314.44310185185</v>
+        <v>46314.3778125</v>
       </c>
       <c r="K48" s="3">
-        <v>100.32289999999999</v>
+        <v>58.06751666666666</v>
       </c>
       <c r="L48" s="2">
-        <v>13.363789</v>
+        <v>9.519687</v>
       </c>
       <c r="M48" s="2">
-        <v>13.363789</v>
+        <v>9.519686</v>
       </c>
       <c r="N48" s="2">
         <v>0</v>
       </c>
       <c r="O48" s="1">
-        <v>478</v>
+        <v>33</v>
       </c>
       <c r="P48" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q48" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R48" s="1">
-        <v>954.0</v>
+        <v>528.0</v>
       </c>
       <c r="S48" s="1">
-        <v>905505.0</v>
+        <v>564432.0</v>
       </c>
       <c r="T48" s="1">
-        <v>202004019.0</v>
+        <v>41322323.0</v>
       </c>
       <c r="U48" s="1">
-        <v>1311783.0</v>
+        <v>971256.0</v>
       </c>
       <c r="V48" s="1">
-        <v>965871</v>
+        <v>132839</v>
+      </c>
+      <c r="W48" s="1">
+        <v>445527</v>
       </c>
       <c r="X48" t="b">
         <v>1</v>
@@ -55678,49 +55892,49 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="B49" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C49" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D49" s="1">
         <v>1</v>
       </c>
       <c r="E49" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H49" t="b">
         <v>0</v>
       </c>
       <c r="I49" s="4">
-        <v>46314.15934027778</v>
+        <v>46314.59266203704</v>
       </c>
       <c r="J49" s="4">
-        <v>46314.193449074075</v>
+        <v>46314.654490740744</v>
       </c>
       <c r="K49" s="3">
-        <v>49.05461666666667</v>
+        <v>73.2598</v>
       </c>
       <c r="L49" s="2">
-        <v>1.393549</v>
+        <v>9.924175</v>
       </c>
       <c r="M49" s="2">
-        <v>1.393549</v>
+        <v>9.924175</v>
       </c>
       <c r="N49" s="2">
         <v>0</v>
       </c>
       <c r="O49" s="1">
-        <v>218</v>
+        <v>293</v>
       </c>
       <c r="P49" s="1">
         <v>0</v>
@@ -55729,69 +55943,99 @@
         <v>0</v>
       </c>
       <c r="R49" s="1">
-        <v>432.0</v>
+        <v>582.0</v>
       </c>
       <c r="S49" s="1">
-        <v>554729.0</v>
+        <v>644532.0</v>
       </c>
       <c r="T49" s="1">
-        <v>96089496.0</v>
+        <v>151776389.0</v>
       </c>
       <c r="U49" s="1">
-        <v>776230.0</v>
+        <v>884968.0</v>
       </c>
       <c r="V49" s="1">
-        <v>781651</v>
+        <v>884970</v>
       </c>
       <c r="X49" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y49" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z49" t="s">
-        <v>798</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D50" s="1">
         <v>1</v>
       </c>
       <c r="E50" t="s">
-        <v>195</v>
+        <v>431</v>
       </c>
       <c r="F50" t="b">
         <v>0</v>
       </c>
       <c r="G50" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H50" t="b">
         <v>0</v>
       </c>
       <c r="I50" s="4">
-        <v>46314.69179398148</v>
+        <v>46314.159166666665</v>
       </c>
       <c r="J50" s="4">
-        <v>46314.70092592593</v>
+        <v>46314.19351851852</v>
+      </c>
+      <c r="K50" s="3">
+        <v>43.80995</v>
+      </c>
+      <c r="L50" s="2">
+        <v>1.351832</v>
+      </c>
+      <c r="M50" s="2">
+        <v>1.351832</v>
+      </c>
+      <c r="N50" s="2">
+        <v>0</v>
+      </c>
+      <c r="O50" s="1">
+        <v>235</v>
+      </c>
+      <c r="P50" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="1">
+        <v>0</v>
+      </c>
+      <c r="R50" s="1">
+        <v>432.0</v>
+      </c>
+      <c r="S50" s="1">
+        <v>538506.0</v>
+      </c>
+      <c r="T50" s="1">
+        <v>92764505.0</v>
+      </c>
+      <c r="U50" s="1">
+        <v>774455.0</v>
+      </c>
+      <c r="V50" s="1">
+        <v>779876</v>
       </c>
       <c r="X50" t="b">
         <v>0</v>
       </c>
       <c r="Y50" t="s">
-        <v>196</v>
+        <v>432</v>
       </c>
       <c r="Z50" t="s">
-        <v>800</v>
+        <v>748</v>
       </c>
     </row>
     <row r="51">
@@ -55799,10 +56043,10 @@
         <v>801</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C51" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D51" s="1">
         <v>2</v>
@@ -55811,34 +56055,34 @@
         <v>110</v>
       </c>
       <c r="F51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" s="4">
-        <v>46314.25201388889</v>
+        <v>46314.21072916667</v>
       </c>
       <c r="J51" s="4">
-        <v>46314.32546296297</v>
+        <v>46314.29785879629</v>
       </c>
       <c r="K51" s="3">
-        <v>95.18496666666667</v>
+        <v>99.19116666666667</v>
       </c>
       <c r="L51" s="2">
-        <v>10.606161</v>
+        <v>14.433891</v>
       </c>
       <c r="M51" s="2">
-        <v>10.606161</v>
+        <v>14.433891</v>
       </c>
       <c r="N51" s="2">
         <v>0</v>
       </c>
       <c r="O51" s="1">
-        <v>335</v>
+        <v>182</v>
       </c>
       <c r="P51" s="1">
         <v>0</v>
@@ -55847,19 +56091,19 @@
         <v>1</v>
       </c>
       <c r="R51" s="1">
-        <v>664.0</v>
+        <v>944.0</v>
       </c>
       <c r="S51" s="1">
-        <v>697439.0</v>
+        <v>719044.0</v>
       </c>
       <c r="T51" s="1">
-        <v>162927364.0</v>
+        <v>235843525.0</v>
       </c>
       <c r="U51" s="1">
-        <v>1051279.0</v>
+        <v>1151474.0</v>
       </c>
       <c r="V51" s="1">
-        <v>965009</v>
+        <v>963737</v>
       </c>
       <c r="X51" t="b">
         <v>1</v>
@@ -55870,10 +56114,10 @@
         <v>802</v>
       </c>
       <c r="B52" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D52" s="1">
         <v>3</v>
@@ -55891,49 +56135,527 @@
         <v>1</v>
       </c>
       <c r="I52" s="4">
+        <v>46314.354363425926</v>
+      </c>
+      <c r="J52" s="4">
+        <v>46314.44310185185</v>
+      </c>
+      <c r="K52" s="3">
+        <v>100.32289999999999</v>
+      </c>
+      <c r="L52" s="2">
+        <v>13.363789</v>
+      </c>
+      <c r="M52" s="2">
+        <v>13.363789</v>
+      </c>
+      <c r="N52" s="2">
+        <v>0</v>
+      </c>
+      <c r="O52" s="1">
+        <v>478</v>
+      </c>
+      <c r="P52" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="1">
+        <v>1</v>
+      </c>
+      <c r="R52" s="1">
+        <v>954.0</v>
+      </c>
+      <c r="S52" s="1">
+        <v>905505.0</v>
+      </c>
+      <c r="T52" s="1">
+        <v>202004019.0</v>
+      </c>
+      <c r="U52" s="1">
+        <v>1311783.0</v>
+      </c>
+      <c r="V52" s="1">
+        <v>965871</v>
+      </c>
+      <c r="X52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>803</v>
+      </c>
+      <c r="B53" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" t="s">
+        <v>74</v>
+      </c>
+      <c r="D53" s="1">
+        <v>1</v>
+      </c>
+      <c r="E53" t="s">
+        <v>431</v>
+      </c>
+      <c r="F53" t="b">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1">
+        <v>1</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4">
+        <v>46314.15934027778</v>
+      </c>
+      <c r="J53" s="4">
+        <v>46314.193449074075</v>
+      </c>
+      <c r="K53" s="3">
+        <v>49.05461666666667</v>
+      </c>
+      <c r="L53" s="2">
+        <v>1.393549</v>
+      </c>
+      <c r="M53" s="2">
+        <v>1.393549</v>
+      </c>
+      <c r="N53" s="2">
+        <v>0</v>
+      </c>
+      <c r="O53" s="1">
+        <v>218</v>
+      </c>
+      <c r="P53" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="1">
+        <v>0</v>
+      </c>
+      <c r="R53" s="1">
+        <v>432.0</v>
+      </c>
+      <c r="S53" s="1">
+        <v>554729.0</v>
+      </c>
+      <c r="T53" s="1">
+        <v>96089496.0</v>
+      </c>
+      <c r="U53" s="1">
+        <v>776230.0</v>
+      </c>
+      <c r="V53" s="1">
+        <v>781651</v>
+      </c>
+      <c r="X53" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y53" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z53" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>805</v>
+      </c>
+      <c r="B54" t="s">
+        <v>73</v>
+      </c>
+      <c r="C54" t="s">
+        <v>74</v>
+      </c>
+      <c r="D54" s="1">
+        <v>1</v>
+      </c>
+      <c r="E54" t="s">
+        <v>195</v>
+      </c>
+      <c r="F54" t="b">
+        <v>0</v>
+      </c>
+      <c r="G54" s="1">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4">
+        <v>46314.69179398148</v>
+      </c>
+      <c r="J54" s="4">
+        <v>46314.70092592593</v>
+      </c>
+      <c r="X54" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y54" t="s">
+        <v>196</v>
+      </c>
+      <c r="Z54" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>807</v>
+      </c>
+      <c r="B55" t="s">
+        <v>73</v>
+      </c>
+      <c r="C55" t="s">
+        <v>74</v>
+      </c>
+      <c r="D55" s="1">
+        <v>2</v>
+      </c>
+      <c r="E55" t="s">
+        <v>110</v>
+      </c>
+      <c r="F55" t="b">
+        <v>1</v>
+      </c>
+      <c r="G55" s="1">
+        <v>2</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4">
+        <v>46314.25201388889</v>
+      </c>
+      <c r="J55" s="4">
+        <v>46314.32546296297</v>
+      </c>
+      <c r="K55" s="3">
+        <v>95.18496666666667</v>
+      </c>
+      <c r="L55" s="2">
+        <v>10.606161</v>
+      </c>
+      <c r="M55" s="2">
+        <v>10.606161</v>
+      </c>
+      <c r="N55" s="2">
+        <v>0</v>
+      </c>
+      <c r="O55" s="1">
+        <v>335</v>
+      </c>
+      <c r="P55" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="1">
+        <v>1</v>
+      </c>
+      <c r="R55" s="1">
+        <v>664.0</v>
+      </c>
+      <c r="S55" s="1">
+        <v>697439.0</v>
+      </c>
+      <c r="T55" s="1">
+        <v>162927364.0</v>
+      </c>
+      <c r="U55" s="1">
+        <v>1051279.0</v>
+      </c>
+      <c r="V55" s="1">
+        <v>965009</v>
+      </c>
+      <c r="X55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>808</v>
+      </c>
+      <c r="B56" t="s">
+        <v>73</v>
+      </c>
+      <c r="C56" t="s">
+        <v>74</v>
+      </c>
+      <c r="D56" s="1">
+        <v>3</v>
+      </c>
+      <c r="E56" t="s">
+        <v>110</v>
+      </c>
+      <c r="F56" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1">
+        <v>5</v>
+      </c>
+      <c r="H56" t="b">
+        <v>1</v>
+      </c>
+      <c r="I56" s="4">
         <v>46314.354537037034</v>
       </c>
-      <c r="J52" s="4">
+      <c r="J56" s="4">
         <v>46314.44809027778</v>
       </c>
-      <c r="K52" s="3">
+      <c r="K56" s="3">
         <v>108.24491666666667</v>
       </c>
-      <c r="L52" s="2">
+      <c r="L56" s="2">
         <v>13.553072</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M56" s="2">
         <v>13.553072</v>
       </c>
-      <c r="N52" s="2">
-        <v>0</v>
-      </c>
-      <c r="O52" s="1">
+      <c r="N56" s="2">
+        <v>0</v>
+      </c>
+      <c r="O56" s="1">
         <v>321</v>
       </c>
-      <c r="P52" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q52" s="1">
-        <v>1</v>
-      </c>
-      <c r="R52" s="1">
+      <c r="P56" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="1">
+        <v>1</v>
+      </c>
+      <c r="R56" s="1">
         <v>934.0</v>
       </c>
-      <c r="S52" s="1">
+      <c r="S56" s="1">
         <v>907702.0</v>
       </c>
-      <c r="T52" s="1">
+      <c r="T56" s="1">
         <v>203600498.0</v>
       </c>
-      <c r="U52" s="1">
+      <c r="U56" s="1">
         <v>1342643.0</v>
       </c>
-      <c r="V52" s="1">
+      <c r="V56" s="1">
         <v>964812</v>
       </c>
-      <c r="X52" t="b">
-        <v>1</v>
+      <c r="X56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>809</v>
+      </c>
+      <c r="B57" t="s">
+        <v>79</v>
+      </c>
+      <c r="C57" t="s">
+        <v>80</v>
+      </c>
+      <c r="D57" s="1">
+        <v>1</v>
+      </c>
+      <c r="E57" t="s">
+        <v>110</v>
+      </c>
+      <c r="F57" t="b">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1">
+        <v>1</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" s="4">
+        <v>46315.19510416667</v>
+      </c>
+      <c r="J57" s="4">
+        <v>46315.23210648148</v>
+      </c>
+      <c r="K57" s="3">
+        <v>47.0307</v>
+      </c>
+      <c r="L57" s="2">
+        <v>7.028553</v>
+      </c>
+      <c r="M57" s="2">
+        <v>2.251192</v>
+      </c>
+      <c r="N57" s="2">
+        <v>4.777361</v>
+      </c>
+      <c r="O57" s="1">
+        <v>14</v>
+      </c>
+      <c r="P57" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q57" s="1">
+        <v>0</v>
+      </c>
+      <c r="R57" s="1">
+        <v>671679.0</v>
+      </c>
+      <c r="S57" s="1">
+        <v>201151.0</v>
+      </c>
+      <c r="T57" s="1">
+        <v>21039932.0</v>
+      </c>
+      <c r="U57" s="1">
+        <v>111024.0</v>
+      </c>
+      <c r="V57" s="1">
+        <v>111026</v>
+      </c>
+      <c r="W57" s="1">
+        <v>186027</v>
+      </c>
+      <c r="X57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>810</v>
+      </c>
+      <c r="B58" t="s">
+        <v>79</v>
+      </c>
+      <c r="C58" t="s">
+        <v>80</v>
+      </c>
+      <c r="D58" s="1">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>777</v>
+      </c>
+      <c r="F58" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1">
+        <v>0</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" s="4">
+        <v>46315.23091435185</v>
+      </c>
+      <c r="X58" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y58" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>811</v>
+      </c>
+      <c r="B59" t="s">
+        <v>81</v>
+      </c>
+      <c r="C59" t="s">
+        <v>82</v>
+      </c>
+      <c r="D59" s="1">
+        <v>1</v>
+      </c>
+      <c r="E59" t="s">
+        <v>110</v>
+      </c>
+      <c r="F59" t="b">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1">
+        <v>1</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" s="4">
+        <v>46315.195289351854</v>
+      </c>
+      <c r="J59" s="4">
+        <v>46315.22857638889</v>
+      </c>
+      <c r="K59" s="3">
+        <v>41.971066666666665</v>
+      </c>
+      <c r="L59" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="M59" s="2">
+        <v>8.729592</v>
+      </c>
+      <c r="N59" s="2">
+        <v>1.605688</v>
+      </c>
+      <c r="O59" s="1">
+        <v>99</v>
+      </c>
+      <c r="P59" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q59" s="1">
+        <v>0</v>
+      </c>
+      <c r="R59" s="1">
+        <v>236477.0</v>
+      </c>
+      <c r="S59" s="1">
+        <v>202289.0</v>
+      </c>
+      <c r="T59" s="1">
+        <v>23194760.0</v>
+      </c>
+      <c r="U59" s="1">
+        <v>288791.0</v>
+      </c>
+      <c r="V59" s="1">
+        <v>294098</v>
+      </c>
+      <c r="W59" s="1">
+        <v>126892</v>
+      </c>
+      <c r="X59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>812</v>
+      </c>
+      <c r="B60" t="s">
+        <v>81</v>
+      </c>
+      <c r="C60" t="s">
+        <v>82</v>
+      </c>
+      <c r="D60" s="1">
+        <v>2</v>
+      </c>
+      <c r="E60" t="s">
+        <v>777</v>
+      </c>
+      <c r="F60" t="b">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" s="4">
+        <v>46315.232256944444</v>
+      </c>
+      <c r="X60" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y60" t="s">
+        <v>778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results: supersede every run on the original Task 4 pack
Task 4 is redone from scratch on the corrected pack (finalists A11, A14,
A21, A22); the workbook's Task 4 sheets now hold only the new runs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/results/experiment-a-results.xlsx
+++ b/docs/results/experiment-a-results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3155" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3166" uniqueCount="838">
   <si>
     <t xml:space="preserve">Experiment results workbook</t>
   </si>
@@ -33,13 +33,13 @@
     <t xml:space="preserve">Cost scenario: billed (all USD columns). Claude USD and Codex USD split the scenario's per-model cost; models whose name starts with gpt are Codex, all others are Claude.</t>
   </si>
   <si>
-    <t xml:space="preserve">Superseded runs excluded using: docs/results/superseded.json (28 listed)</t>
+    <t xml:space="preserve">Superseded runs excluded using: docs/results/superseded.json (53 listed)</t>
   </si>
   <si>
     <t xml:space="preserve">Statuses dropped: cli_error, running, stopped, usage_limit</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 29 of 59 attempts in the results</t>
+    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 4 of 59 attempts in the results</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -2250,12 +2250,21 @@
     <t xml:space="preserve">d30af6eb</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A1 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">e77f9343</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A1 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">b84c3e90</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A1 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">2f6bd8eb</t>
   </si>
   <si>
@@ -2274,6 +2283,9 @@
     <t xml:space="preserve">dfd2359b</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A2 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">0df855ac</t>
   </si>
   <si>
@@ -2295,15 +2307,24 @@
     <t xml:space="preserve">52d7d848</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A2 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">76771788</t>
   </si>
   <si>
     <t xml:space="preserve">5af65ea5</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A4 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">4dbd1845</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A4 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">59986a93</t>
   </si>
   <si>
@@ -2322,6 +2343,9 @@
     <t xml:space="preserve">66f31f60</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A4 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">98cbe722</t>
   </si>
   <si>
@@ -2340,6 +2364,9 @@
     <t xml:space="preserve">f6294287</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A11 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">c77fc1a9</t>
   </si>
   <si>
@@ -2349,6 +2376,9 @@
     <t xml:space="preserve">ee0e6aeb</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A11 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">f305c31e</t>
   </si>
   <si>
@@ -2361,6 +2391,9 @@
     <t xml:space="preserve">dd4497e8</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A11 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">0d3109e9</t>
   </si>
   <si>
@@ -2370,12 +2403,21 @@
     <t xml:space="preserve">d0c40df1</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A12 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">4523a58d</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A12 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">4457436e</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A12 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">2aef8aff</t>
   </si>
   <si>
@@ -2388,18 +2430,27 @@
     <t xml:space="preserve">65d92f15</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A14 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">e56ed8a8</t>
   </si>
   <si>
     <t xml:space="preserve">6536e57a</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A14 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">e8c4f691</t>
   </si>
   <si>
     <t xml:space="preserve">7137e856</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A14 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">0c38b8d3</t>
   </si>
   <si>
@@ -2412,24 +2463,42 @@
     <t xml:space="preserve">af89e08e</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A15 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">67702480</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A15 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">1cd24f63</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A15 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">9c1cb7d2</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A16 task4 rep 1: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">da8823c0</t>
   </si>
   <si>
     <t xml:space="preserve">b267119a</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A16 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">b33bb6ba</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A16 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">5fb731e0</t>
   </si>
   <si>
@@ -2445,7 +2514,13 @@
     <t xml:space="preserve">d768c362</t>
   </si>
   <si>
+    <t xml:space="preserve">superseded: A17 task4 rep 2: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
+  </si>
+  <si>
     <t xml:space="preserve">a5775bc0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">superseded: A17 task4 rep 3: run on the original Task 4 pack, whose stub-vs-real-cFS defects decided pass/fail; Task 4 is redone from scratch on the corrected pack</t>
   </si>
   <si>
     <t xml:space="preserve">1dbd8ee4</t>
@@ -2731,8 +2806,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC12" totalsRowShown="0">
-  <autoFilter ref="A1:AC12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC5" totalsRowShown="0">
+  <autoFilter ref="A1:AC5"/>
   <tableColumns count="29">
     <tableColumn id="1" name="Arm"/>
     <tableColumn id="2" name="Description"/>
@@ -51232,7 +51307,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC12"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -51357,73 +51432,70 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C2" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2">
-        <v>20.747254333333334</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1.0</v>
+        <v>12.116333</v>
       </c>
       <c r="G2" s="2">
-        <v>62.241763</v>
+        <v>12.116333</v>
       </c>
       <c r="H2" s="2">
-        <v>18.230683</v>
+        <v>12.116333</v>
       </c>
       <c r="I2" s="2">
-        <v>21.32055</v>
+        <v>12.116333</v>
       </c>
       <c r="J2" s="2">
-        <v>22.69053</v>
+        <v>12.116333</v>
       </c>
       <c r="K2" s="2">
-        <v>4.459847</v>
+        <v>0.0</v>
       </c>
       <c r="L2" s="2">
-        <v>21.32055</v>
+        <v>12.116332</v>
       </c>
       <c r="M2" s="2">
         <v>0</v>
       </c>
       <c r="N2" s="3">
-        <v>59.72193333333333</v>
+        <v>45.978899999999996</v>
       </c>
       <c r="O2" s="3">
-        <v>67.27728333333333</v>
+        <v>45.978899999999996</v>
       </c>
       <c r="P2" s="3">
-        <v>70.25485</v>
+        <v>45.978899999999996</v>
       </c>
       <c r="Q2" s="1">
-        <v>171</v>
+        <v>18</v>
       </c>
       <c r="R2" s="1">
-        <v>194</v>
+        <v>18</v>
       </c>
       <c r="S2" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T2" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W2" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X2" s="1">
         <v>0</v>
@@ -51432,81 +51504,84 @@
         <v>0</v>
       </c>
       <c r="Z2" s="3">
-        <v>474.089</v>
+        <v>405.401</v>
       </c>
       <c r="AA2" s="3">
-        <v>549.187</v>
+        <v>405.401</v>
+      </c>
+      <c r="AB2" s="3">
+        <v>371.552</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>371.552</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="C3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2">
-        <v>33.0455725</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1.5927684680139924</v>
+        <v>6.656134</v>
       </c>
       <c r="G3" s="2">
-        <v>66.091145</v>
+        <v>6.656134</v>
       </c>
       <c r="H3" s="2">
-        <v>32.8281</v>
+        <v>6.656134</v>
       </c>
       <c r="I3" s="2">
-        <v>33.0455725</v>
+        <v>6.656134</v>
       </c>
       <c r="J3" s="2">
-        <v>33.263045</v>
+        <v>6.656134</v>
       </c>
       <c r="K3" s="2">
-        <v>0.434944999999999</v>
+        <v>0.0</v>
       </c>
       <c r="L3" s="2">
-        <v>33.0455725</v>
+        <v>6.656134</v>
       </c>
       <c r="M3" s="2">
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N3" s="3">
-        <v>67.2674</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="O3" s="3">
-        <v>78.40260833333333</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="P3" s="3">
-        <v>89.53781666666667</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="Q3" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="R3" s="1">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="S3" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="T3" s="1">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="U3" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V3" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W3" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X3" s="1">
         <v>0</v>
@@ -51515,87 +51590,84 @@
         <v>0</v>
       </c>
       <c r="Z3" s="3">
-        <v>170.786</v>
+        <v>44.805</v>
       </c>
       <c r="AA3" s="3">
-        <v>194.384</v>
+        <v>44.805</v>
       </c>
       <c r="AB3" s="3">
-        <v>245.496</v>
+        <v>506.67</v>
       </c>
       <c r="AC3" s="3">
-        <v>279.819</v>
+        <v>506.67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2">
-        <v>14.328286999999998</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.6906112379882298</v>
+        <v>7.028553</v>
       </c>
       <c r="G4" s="2">
-        <v>42.984860999999995</v>
+        <v>7.028553</v>
       </c>
       <c r="H4" s="2">
-        <v>10.490442</v>
+        <v>7.028553</v>
       </c>
       <c r="I4" s="2">
-        <v>15.348486</v>
+        <v>7.028553</v>
       </c>
       <c r="J4" s="2">
-        <v>17.145933</v>
+        <v>7.028553</v>
       </c>
       <c r="K4" s="2">
-        <v>6.655491</v>
+        <v>0.0</v>
       </c>
       <c r="L4" s="2">
-        <v>15.348486999999999</v>
+        <v>2.251192</v>
       </c>
       <c r="M4" s="2">
-        <v>0</v>
+        <v>4.777361</v>
       </c>
       <c r="N4" s="3">
-        <v>55.542183333333334</v>
+        <v>47.0307</v>
       </c>
       <c r="O4" s="3">
-        <v>63.47421666666666</v>
+        <v>47.0307</v>
       </c>
       <c r="P4" s="3">
-        <v>67.94765</v>
+        <v>47.0307</v>
       </c>
       <c r="Q4" s="1">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="R4" s="1">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="S4" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T4" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="U4" s="1">
         <v>1</v>
       </c>
       <c r="V4" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W4" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -51604,87 +51676,84 @@
         <v>0</v>
       </c>
       <c r="Z4" s="3">
-        <v>133.032</v>
+        <v>111.026</v>
       </c>
       <c r="AA4" s="3">
-        <v>226.373</v>
+        <v>111.026</v>
       </c>
       <c r="AB4" s="3">
-        <v>162.267</v>
+        <v>186.027</v>
       </c>
       <c r="AC4" s="3">
-        <v>258.548</v>
+        <v>186.027</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="C5" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2">
-        <v>13.662117</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0.6585024109937245</v>
+        <v>10.33528</v>
       </c>
       <c r="G5" s="2">
-        <v>40.986351</v>
+        <v>10.33528</v>
       </c>
       <c r="H5" s="2">
-        <v>8.11915</v>
+        <v>10.33528</v>
       </c>
       <c r="I5" s="2">
-        <v>10.375434</v>
+        <v>10.33528</v>
       </c>
       <c r="J5" s="2">
-        <v>12.116333</v>
+        <v>10.33528</v>
       </c>
       <c r="K5" s="2">
-        <v>3.9971829999999997</v>
+        <v>0.0</v>
       </c>
       <c r="L5" s="2">
-        <v>10.375434</v>
+        <v>8.729592</v>
       </c>
       <c r="M5" s="2">
-        <v>0.0</v>
+        <v>1.605688</v>
       </c>
       <c r="N5" s="3">
-        <v>37.165499999999994</v>
+        <v>41.971066666666665</v>
       </c>
       <c r="O5" s="3">
-        <v>42.74603333333333</v>
+        <v>41.971066666666665</v>
       </c>
       <c r="P5" s="3">
-        <v>200.98263333333335</v>
+        <v>41.971066666666665</v>
       </c>
       <c r="Q5" s="1">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="R5" s="1">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="S5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T5" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="U5" s="1">
         <v>1</v>
       </c>
       <c r="V5" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W5" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X5" s="1">
         <v>0</v>
@@ -51693,620 +51762,15 @@
         <v>0</v>
       </c>
       <c r="Z5" s="3">
-        <v>293.858</v>
+        <v>294.098</v>
       </c>
       <c r="AA5" s="3">
-        <v>458.412</v>
+        <v>294.098</v>
       </c>
       <c r="AB5" s="3">
-        <v>322.948</v>
+        <v>126.892</v>
       </c>
       <c r="AC5" s="3">
-        <v>477.389</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1">
-        <v>3</v>
-      </c>
-      <c r="E6" s="2">
-        <v>20.852458000000002</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1.005070727190038</v>
-      </c>
-      <c r="G6" s="2">
-        <v>41.704916000000004</v>
-      </c>
-      <c r="H6" s="2">
-        <v>9.165487</v>
-      </c>
-      <c r="I6" s="2">
-        <v>11.371427</v>
-      </c>
-      <c r="J6" s="2">
-        <v>21.168002</v>
-      </c>
-      <c r="K6" s="2">
-        <v>12.002515</v>
-      </c>
-      <c r="L6" s="2">
-        <v>11.371427</v>
-      </c>
-      <c r="M6" s="2">
-        <v>0</v>
-      </c>
-      <c r="N6" s="3">
-        <v>48.04756666666666</v>
-      </c>
-      <c r="O6" s="3">
-        <v>50.72746666666667</v>
-      </c>
-      <c r="P6" s="3">
-        <v>104.91581666666666</v>
-      </c>
-      <c r="Q6" s="1">
-        <v>98</v>
-      </c>
-      <c r="R6" s="1">
-        <v>178</v>
-      </c>
-      <c r="S6" s="1">
-        <v>0</v>
-      </c>
-      <c r="T6" s="1">
-        <v>0</v>
-      </c>
-      <c r="U6" s="1">
-        <v>1</v>
-      </c>
-      <c r="V6" s="1">
-        <v>5</v>
-      </c>
-      <c r="W6" s="1">
-        <v>2</v>
-      </c>
-      <c r="X6" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="3">
-        <v>498.624</v>
-      </c>
-      <c r="AA6" s="3">
-        <v>764.579</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="1">
-        <v>4</v>
-      </c>
-      <c r="D7" s="1">
-        <v>4</v>
-      </c>
-      <c r="E7" s="2">
-        <v>7.28428675</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0.3510964213851076</v>
-      </c>
-      <c r="G7" s="2">
-        <v>29.137147</v>
-      </c>
-      <c r="H7" s="2">
-        <v>5.548321</v>
-      </c>
-      <c r="I7" s="2">
-        <v>7.527323</v>
-      </c>
-      <c r="J7" s="2">
-        <v>8.53418</v>
-      </c>
-      <c r="K7" s="2">
-        <v>2.9858589999999996</v>
-      </c>
-      <c r="L7" s="2">
-        <v>7.527323</v>
-      </c>
-      <c r="M7" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="N7" s="3">
-        <v>44.932900000000004</v>
-      </c>
-      <c r="O7" s="3">
-        <v>57.42019166666667</v>
-      </c>
-      <c r="P7" s="3">
-        <v>60.036500000000004</v>
-      </c>
-      <c r="Q7" s="1">
-        <v>4</v>
-      </c>
-      <c r="R7" s="1">
-        <v>32</v>
-      </c>
-      <c r="S7" s="1">
-        <v>3</v>
-      </c>
-      <c r="T7" s="1">
-        <v>7</v>
-      </c>
-      <c r="U7" s="1">
-        <v>1</v>
-      </c>
-      <c r="V7" s="1">
-        <v>3</v>
-      </c>
-      <c r="W7" s="1">
-        <v>3</v>
-      </c>
-      <c r="X7" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="3">
-        <v>44.805</v>
-      </c>
-      <c r="AA7" s="3">
-        <v>81.975</v>
-      </c>
-      <c r="AB7" s="3">
-        <v>299.031</v>
-      </c>
-      <c r="AC7" s="3">
-        <v>506.67</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="1">
-        <v>3</v>
-      </c>
-      <c r="D8" s="1">
-        <v>3</v>
-      </c>
-      <c r="E8" s="2">
-        <v>10.894769333333334</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.5251186088671685</v>
-      </c>
-      <c r="G8" s="2">
-        <v>32.684308</v>
-      </c>
-      <c r="H8" s="2">
-        <v>9.519687</v>
-      </c>
-      <c r="I8" s="2">
-        <v>10.446109</v>
-      </c>
-      <c r="J8" s="2">
-        <v>12.718512</v>
-      </c>
-      <c r="K8" s="2">
-        <v>3.198825000000001</v>
-      </c>
-      <c r="L8" s="2">
-        <v>10.446109</v>
-      </c>
-      <c r="M8" s="2">
-        <v>0</v>
-      </c>
-      <c r="N8" s="3">
-        <v>48.78155</v>
-      </c>
-      <c r="O8" s="3">
-        <v>58.06751666666666</v>
-      </c>
-      <c r="P8" s="3">
-        <v>65.17911666666666</v>
-      </c>
-      <c r="Q8" s="1">
-        <v>33</v>
-      </c>
-      <c r="R8" s="1">
-        <v>51</v>
-      </c>
-      <c r="S8" s="1">
-        <v>3</v>
-      </c>
-      <c r="T8" s="1">
-        <v>6</v>
-      </c>
-      <c r="U8" s="1">
-        <v>2</v>
-      </c>
-      <c r="V8" s="1">
-        <v>3</v>
-      </c>
-      <c r="W8" s="1">
-        <v>3</v>
-      </c>
-      <c r="X8" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="3">
-        <v>132.839</v>
-      </c>
-      <c r="AA8" s="3">
-        <v>223.412</v>
-      </c>
-      <c r="AB8" s="3">
-        <v>358.765</v>
-      </c>
-      <c r="AC8" s="3">
-        <v>445.527</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" s="1">
-        <v>3</v>
-      </c>
-      <c r="E9" s="2">
-        <v>37.721855</v>
-      </c>
-      <c r="F9" s="2">
-        <v>1.8181613043319482</v>
-      </c>
-      <c r="G9" s="2">
-        <v>37.721855</v>
-      </c>
-      <c r="H9" s="2">
-        <v>9.924175</v>
-      </c>
-      <c r="I9" s="2">
-        <v>13.363789</v>
-      </c>
-      <c r="J9" s="2">
-        <v>14.433891</v>
-      </c>
-      <c r="K9" s="2">
-        <v>4.509715999999999</v>
-      </c>
-      <c r="L9" s="2">
-        <v>13.363789</v>
-      </c>
-      <c r="M9" s="2">
-        <v>0</v>
-      </c>
-      <c r="N9" s="3">
-        <v>73.2598</v>
-      </c>
-      <c r="O9" s="3">
-        <v>99.19116666666667</v>
-      </c>
-      <c r="P9" s="3">
-        <v>100.32289999999999</v>
-      </c>
-      <c r="Q9" s="1">
-        <v>182</v>
-      </c>
-      <c r="R9" s="1">
-        <v>478</v>
-      </c>
-      <c r="S9" s="1">
-        <v>0</v>
-      </c>
-      <c r="T9" s="1">
-        <v>0</v>
-      </c>
-      <c r="U9" s="1">
-        <v>3</v>
-      </c>
-      <c r="V9" s="1">
-        <v>5</v>
-      </c>
-      <c r="W9" s="1">
-        <v>3</v>
-      </c>
-      <c r="X9" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="1">
-        <v>1</v>
-      </c>
-      <c r="Z9" s="3">
-        <v>884.97</v>
-      </c>
-      <c r="AA9" s="3">
-        <v>965.871</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1">
-        <v>2</v>
-      </c>
-      <c r="E10" s="2">
-        <v>24.159233</v>
-      </c>
-      <c r="F10" s="2">
-        <v>1.1644544676538162</v>
-      </c>
-      <c r="G10" s="2">
-        <v>24.159233</v>
-      </c>
-      <c r="H10" s="2">
-        <v>10.606161</v>
-      </c>
-      <c r="I10" s="2">
-        <v>12.0796165</v>
-      </c>
-      <c r="J10" s="2">
-        <v>13.553072</v>
-      </c>
-      <c r="K10" s="2">
-        <v>2.946911</v>
-      </c>
-      <c r="L10" s="2">
-        <v>12.0796165</v>
-      </c>
-      <c r="M10" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="N10" s="3">
-        <v>95.18496666666667</v>
-      </c>
-      <c r="O10" s="3">
-        <v>101.71494166666668</v>
-      </c>
-      <c r="P10" s="3">
-        <v>108.24491666666667</v>
-      </c>
-      <c r="Q10" s="1">
-        <v>321</v>
-      </c>
-      <c r="R10" s="1">
-        <v>335</v>
-      </c>
-      <c r="S10" s="1">
-        <v>0</v>
-      </c>
-      <c r="T10" s="1">
-        <v>0</v>
-      </c>
-      <c r="U10" s="1">
-        <v>2</v>
-      </c>
-      <c r="V10" s="1">
-        <v>5</v>
-      </c>
-      <c r="W10" s="1">
-        <v>2</v>
-      </c>
-      <c r="X10" s="1">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="1">
-        <v>1</v>
-      </c>
-      <c r="Z10" s="3">
-        <v>964.812</v>
-      </c>
-      <c r="AA10" s="3">
-        <v>965.009</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1">
-        <v>1</v>
-      </c>
-      <c r="E11" s="2">
-        <v>7.028553</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.33877027230093076</v>
-      </c>
-      <c r="G11" s="2">
-        <v>7.028553</v>
-      </c>
-      <c r="H11" s="2">
-        <v>7.028553</v>
-      </c>
-      <c r="I11" s="2">
-        <v>7.028553</v>
-      </c>
-      <c r="J11" s="2">
-        <v>7.028553</v>
-      </c>
-      <c r="K11" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="L11" s="2">
-        <v>2.251192</v>
-      </c>
-      <c r="M11" s="2">
-        <v>4.777361</v>
-      </c>
-      <c r="N11" s="3">
-        <v>47.0307</v>
-      </c>
-      <c r="O11" s="3">
-        <v>47.0307</v>
-      </c>
-      <c r="P11" s="3">
-        <v>47.0307</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>14</v>
-      </c>
-      <c r="R11" s="1">
-        <v>14</v>
-      </c>
-      <c r="S11" s="1">
-        <v>6</v>
-      </c>
-      <c r="T11" s="1">
-        <v>6</v>
-      </c>
-      <c r="U11" s="1">
-        <v>1</v>
-      </c>
-      <c r="V11" s="1">
-        <v>1</v>
-      </c>
-      <c r="W11" s="1">
-        <v>0</v>
-      </c>
-      <c r="X11" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="3">
-        <v>111.026</v>
-      </c>
-      <c r="AA11" s="3">
-        <v>111.026</v>
-      </c>
-      <c r="AB11" s="3">
-        <v>186.027</v>
-      </c>
-      <c r="AC11" s="3">
-        <v>186.027</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2">
-        <v>10.33528</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0.4981516992055639</v>
-      </c>
-      <c r="G12" s="2">
-        <v>10.33528</v>
-      </c>
-      <c r="H12" s="2">
-        <v>10.33528</v>
-      </c>
-      <c r="I12" s="2">
-        <v>10.33528</v>
-      </c>
-      <c r="J12" s="2">
-        <v>10.33528</v>
-      </c>
-      <c r="K12" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="L12" s="2">
-        <v>8.729592</v>
-      </c>
-      <c r="M12" s="2">
-        <v>1.605688</v>
-      </c>
-      <c r="N12" s="3">
-        <v>41.971066666666665</v>
-      </c>
-      <c r="O12" s="3">
-        <v>41.971066666666665</v>
-      </c>
-      <c r="P12" s="3">
-        <v>41.971066666666665</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>99</v>
-      </c>
-      <c r="R12" s="1">
-        <v>99</v>
-      </c>
-      <c r="S12" s="1">
-        <v>2</v>
-      </c>
-      <c r="T12" s="1">
-        <v>2</v>
-      </c>
-      <c r="U12" s="1">
-        <v>1</v>
-      </c>
-      <c r="V12" s="1">
-        <v>1</v>
-      </c>
-      <c r="W12" s="1">
-        <v>0</v>
-      </c>
-      <c r="X12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="3">
-        <v>294.098</v>
-      </c>
-      <c r="AA12" s="3">
-        <v>294.098</v>
-      </c>
-      <c r="AB12" s="3">
-        <v>126.892</v>
-      </c>
-      <c r="AC12" s="3">
         <v>126.892</v>
       </c>
     </row>
@@ -52346,7 +51810,7 @@
     <col min="22" max="22" width="24" customWidth="1"/>
     <col min="23" max="23" width="28" customWidth="1"/>
     <col min="24" max="24" width="14" customWidth="1"/>
-    <col min="25" max="25" width="40" customWidth="1"/>
+    <col min="25" max="25" width="60" customWidth="1"/>
     <col min="26" max="26" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -52498,12 +51962,15 @@
         <v>549187</v>
       </c>
       <c r="X2" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>743</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B3" t="s">
         <v>41</v>
@@ -52569,12 +52036,15 @@
         <v>474089</v>
       </c>
       <c r="X3" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>745</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
@@ -52640,12 +52110,15 @@
         <v>542433</v>
       </c>
       <c r="X4" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>747</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="B5" t="s">
         <v>43</v>
@@ -52720,12 +52193,12 @@
         <v>432</v>
       </c>
       <c r="Z5" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="B6" t="s">
         <v>43</v>
@@ -52800,12 +52273,12 @@
         <v>432</v>
       </c>
       <c r="Z6" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="B7" t="s">
         <v>43</v>
@@ -52867,7 +52340,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
@@ -52936,12 +52409,15 @@
         <v>245496</v>
       </c>
       <c r="X8" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>754</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B9" t="s">
         <v>43</v>
@@ -53016,12 +52492,12 @@
         <v>432</v>
       </c>
       <c r="Z9" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B10" t="s">
         <v>43</v>
@@ -53096,12 +52572,12 @@
         <v>432</v>
       </c>
       <c r="Z10" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="B11" t="s">
         <v>43</v>
@@ -53176,12 +52652,12 @@
         <v>196</v>
       </c>
       <c r="Z11" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="B12" t="s">
         <v>43</v>
@@ -53243,7 +52719,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B13" t="s">
         <v>43</v>
@@ -53312,12 +52788,15 @@
         <v>279819</v>
       </c>
       <c r="X13" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>762</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B14" t="s">
         <v>43</v>
@@ -53379,7 +52858,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="B15" t="s">
         <v>47</v>
@@ -53448,12 +52927,15 @@
         <v>258548</v>
       </c>
       <c r="X15" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>765</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="B16" t="s">
         <v>47</v>
@@ -53522,12 +53004,15 @@
         <v>214734</v>
       </c>
       <c r="X16" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>767</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="B17" t="s">
         <v>47</v>
@@ -53602,12 +53087,12 @@
         <v>432</v>
       </c>
       <c r="Z17" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="B18" t="s">
         <v>47</v>
@@ -53682,12 +53167,12 @@
         <v>432</v>
       </c>
       <c r="Z18" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="B19" t="s">
         <v>47</v>
@@ -53762,12 +53247,12 @@
         <v>566</v>
       </c>
       <c r="Z19" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B20" t="s">
         <v>47</v>
@@ -53836,12 +53321,15 @@
         <v>162267</v>
       </c>
       <c r="X20" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>767</v>
+        <v>775</v>
       </c>
       <c r="B21" t="s">
         <v>47</v>
@@ -53916,12 +53404,12 @@
         <v>432</v>
       </c>
       <c r="Z21" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="B22" t="s">
         <v>47</v>
@@ -53996,12 +53484,12 @@
         <v>432</v>
       </c>
       <c r="Z22" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="B23" t="s">
         <v>47</v>
@@ -54076,12 +53564,12 @@
         <v>566</v>
       </c>
       <c r="Z23" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
       <c r="B24" t="s">
         <v>61</v>
@@ -54156,12 +53644,12 @@
         <v>432</v>
       </c>
       <c r="Z24" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="B25" t="s">
         <v>61</v>
@@ -54235,7 +53723,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="B26" t="s">
         <v>61</v>
@@ -54304,12 +53792,15 @@
         <v>362172</v>
       </c>
       <c r="X26" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>781</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>773</v>
+        <v>782</v>
       </c>
       <c r="B27" t="s">
         <v>61</v>
@@ -54384,12 +53875,12 @@
         <v>432</v>
       </c>
       <c r="Z27" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>774</v>
+        <v>783</v>
       </c>
       <c r="B28" t="s">
         <v>61</v>
@@ -54464,12 +53955,12 @@
         <v>432</v>
       </c>
       <c r="Z28" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>775</v>
+        <v>784</v>
       </c>
       <c r="B29" t="s">
         <v>61</v>
@@ -54538,12 +54029,15 @@
         <v>477389</v>
       </c>
       <c r="X29" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>785</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>776</v>
+        <v>786</v>
       </c>
       <c r="B30" t="s">
         <v>61</v>
@@ -54555,7 +54049,7 @@
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
@@ -54573,12 +54067,12 @@
         <v>0</v>
       </c>
       <c r="Y30" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>779</v>
+        <v>789</v>
       </c>
       <c r="B31" t="s">
         <v>61</v>
@@ -54647,12 +54141,15 @@
         <v>322948</v>
       </c>
       <c r="X31" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>790</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="B32" t="s">
         <v>63</v>
@@ -54724,12 +54221,12 @@
         <v>432</v>
       </c>
       <c r="Z32" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
       <c r="B33" t="s">
         <v>63</v>
@@ -54801,12 +54298,12 @@
         <v>432</v>
       </c>
       <c r="Z33" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="B34" t="s">
         <v>63</v>
@@ -54872,12 +54369,15 @@
         <v>559068</v>
       </c>
       <c r="X34" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>783</v>
+        <v>795</v>
       </c>
       <c r="B35" t="s">
         <v>63</v>
@@ -54943,12 +54443,15 @@
         <v>498624</v>
       </c>
       <c r="X35" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>796</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>784</v>
+        <v>797</v>
       </c>
       <c r="B36" t="s">
         <v>63</v>
@@ -55014,12 +54517,15 @@
         <v>764579</v>
       </c>
       <c r="X36" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>798</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>785</v>
+        <v>799</v>
       </c>
       <c r="B37" t="s">
         <v>67</v>
@@ -55094,12 +54600,12 @@
         <v>432</v>
       </c>
       <c r="Z37" t="s">
-        <v>786</v>
+        <v>800</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>787</v>
+        <v>801</v>
       </c>
       <c r="B38" t="s">
         <v>67</v>
@@ -55173,7 +54679,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>788</v>
+        <v>802</v>
       </c>
       <c r="B39" t="s">
         <v>67</v>
@@ -55242,12 +54748,15 @@
         <v>380955</v>
       </c>
       <c r="X39" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>803</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>789</v>
+        <v>804</v>
       </c>
       <c r="B40" t="s">
         <v>67</v>
@@ -55322,12 +54831,12 @@
         <v>432</v>
       </c>
       <c r="Z40" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>790</v>
+        <v>805</v>
       </c>
       <c r="B41" t="s">
         <v>67</v>
@@ -55396,12 +54905,15 @@
         <v>427464</v>
       </c>
       <c r="X41" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>791</v>
+        <v>807</v>
       </c>
       <c r="B42" t="s">
         <v>67</v>
@@ -55413,7 +54925,7 @@
         <v>2</v>
       </c>
       <c r="E42" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="F42" t="b">
         <v>0</v>
@@ -55431,12 +54943,12 @@
         <v>0</v>
       </c>
       <c r="Y42" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>792</v>
+        <v>808</v>
       </c>
       <c r="B43" t="s">
         <v>67</v>
@@ -55505,12 +55017,15 @@
         <v>299031</v>
       </c>
       <c r="X43" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>809</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>793</v>
+        <v>810</v>
       </c>
       <c r="B44" t="s">
         <v>69</v>
@@ -55585,12 +55100,12 @@
         <v>432</v>
       </c>
       <c r="Z44" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>795</v>
+        <v>812</v>
       </c>
       <c r="B45" t="s">
         <v>69</v>
@@ -55665,12 +55180,12 @@
         <v>432</v>
       </c>
       <c r="Z45" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>796</v>
+        <v>813</v>
       </c>
       <c r="B46" t="s">
         <v>69</v>
@@ -55739,12 +55254,15 @@
         <v>420234</v>
       </c>
       <c r="X46" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y46" t="s">
+        <v>814</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>797</v>
+        <v>815</v>
       </c>
       <c r="B47" t="s">
         <v>69</v>
@@ -55813,12 +55331,15 @@
         <v>358765</v>
       </c>
       <c r="X47" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y47" t="s">
+        <v>816</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>798</v>
+        <v>817</v>
       </c>
       <c r="B48" t="s">
         <v>69</v>
@@ -55887,12 +55408,15 @@
         <v>445527</v>
       </c>
       <c r="X48" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y48" t="s">
+        <v>818</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>799</v>
+        <v>819</v>
       </c>
       <c r="B49" t="s">
         <v>71</v>
@@ -55958,12 +55482,15 @@
         <v>884970</v>
       </c>
       <c r="X49" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y49" t="s">
+        <v>820</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>800</v>
+        <v>821</v>
       </c>
       <c r="B50" t="s">
         <v>71</v>
@@ -56035,12 +55562,12 @@
         <v>432</v>
       </c>
       <c r="Z50" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>801</v>
+        <v>822</v>
       </c>
       <c r="B51" t="s">
         <v>71</v>
@@ -56106,12 +55633,15 @@
         <v>963737</v>
       </c>
       <c r="X51" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y51" t="s">
+        <v>823</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>802</v>
+        <v>824</v>
       </c>
       <c r="B52" t="s">
         <v>71</v>
@@ -56177,12 +55707,15 @@
         <v>965871</v>
       </c>
       <c r="X52" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y52" t="s">
+        <v>825</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>803</v>
+        <v>826</v>
       </c>
       <c r="B53" t="s">
         <v>73</v>
@@ -56254,12 +55787,12 @@
         <v>432</v>
       </c>
       <c r="Z53" t="s">
-        <v>804</v>
+        <v>827</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>805</v>
+        <v>828</v>
       </c>
       <c r="B54" t="s">
         <v>73</v>
@@ -56295,12 +55828,12 @@
         <v>196</v>
       </c>
       <c r="Z54" t="s">
-        <v>806</v>
+        <v>829</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>807</v>
+        <v>830</v>
       </c>
       <c r="B55" t="s">
         <v>73</v>
@@ -56366,12 +55899,15 @@
         <v>965009</v>
       </c>
       <c r="X55" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y55" t="s">
+        <v>831</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>808</v>
+        <v>832</v>
       </c>
       <c r="B56" t="s">
         <v>73</v>
@@ -56437,12 +55973,15 @@
         <v>964812</v>
       </c>
       <c r="X56" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y56" t="s">
+        <v>833</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>809</v>
+        <v>834</v>
       </c>
       <c r="B57" t="s">
         <v>79</v>
@@ -56516,7 +56055,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>810</v>
+        <v>835</v>
       </c>
       <c r="B58" t="s">
         <v>79</v>
@@ -56528,7 +56067,7 @@
         <v>2</v>
       </c>
       <c r="E58" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="F58" t="b">
         <v>0</v>
@@ -56546,12 +56085,12 @@
         <v>0</v>
       </c>
       <c r="Y58" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>811</v>
+        <v>836</v>
       </c>
       <c r="B59" t="s">
         <v>81</v>
@@ -56625,7 +56164,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>812</v>
+        <v>837</v>
       </c>
       <c r="B60" t="s">
         <v>81</v>
@@ -56637,7 +56176,7 @@
         <v>2</v>
       </c>
       <c r="E60" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="F60" t="b">
         <v>0</v>
@@ -56655,7 +56194,7 @@
         <v>0</v>
       </c>
       <c r="Y60" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Results: Task 4 on the corrected pack, A11, A14, A21 and A22
All 12 runs passed in round one. Rewrites task4.md, regenerates the
Task 4 charts, drops the old pack's chart note and re-exports the
workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/results/experiment-a-results.xlsx
+++ b/docs/results/experiment-a-results.xlsx
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3166" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3178" uniqueCount="840">
   <si>
     <t xml:space="preserve">Experiment results workbook</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated: 2026-10-20T05:40Z</t>
+    <t xml:space="preserve">Generated: 2026-10-20T07:39:16Z</t>
   </si>
   <si>
     <t xml:space="preserve">Runs directory: /workspace/agent-experiments-matrix</t>
@@ -39,7 +39,7 @@
     <t xml:space="preserve">Statuses dropped: cli_error, running, stopped, usage_limit</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 4 of 59 attempts in the results</t>
+    <t xml:space="preserve">Attempts per task: task1: 210 of 215 attempts in the results; task2: 194 of 209 attempts in the results; task3: 117 of 169 attempts in the results; task4: 12 of 63 attempts in the results</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -2382,10 +2382,7 @@
     <t xml:space="preserve">f305c31e</t>
   </si>
   <si>
-    <t xml:space="preserve">running</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dropped status: running</t>
+    <t xml:space="preserve">afbfddbc</t>
   </si>
   <si>
     <t xml:space="preserve">dd4497e8</t>
@@ -2445,6 +2442,9 @@
     <t xml:space="preserve">e8c4f691</t>
   </si>
   <si>
+    <t xml:space="preserve">4dbb8691</t>
+  </si>
+  <si>
     <t xml:space="preserve">7137e856</t>
   </si>
   <si>
@@ -2529,10 +2529,16 @@
     <t xml:space="preserve">34c1b008</t>
   </si>
   <si>
+    <t xml:space="preserve">3d3ac940</t>
+  </si>
+  <si>
     <t xml:space="preserve">019d4e30</t>
   </si>
   <si>
     <t xml:space="preserve">02411e1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">345ff958</t>
   </si>
 </sst>
 </file>
@@ -2844,8 +2850,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Runs_T4" displayName="Runs_T4" ref="A1:Z60" totalsRowShown="0">
-  <autoFilter ref="A1:Z60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Runs_T4" displayName="Runs_T4" ref="A1:Z64" totalsRowShown="0">
+  <autoFilter ref="A1:Z64"/>
   <tableColumns count="26">
     <tableColumn id="1" name="run_id"/>
     <tableColumn id="2" name="arm"/>
@@ -51438,55 +51444,55 @@
         <v>62</v>
       </c>
       <c r="C2" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" s="2">
-        <v>12.116333</v>
+        <v>10.355836666666667</v>
       </c>
       <c r="G2" s="2">
-        <v>12.116333</v>
+        <v>31.06751</v>
       </c>
       <c r="H2" s="2">
-        <v>12.116333</v>
+        <v>8.204365</v>
       </c>
       <c r="I2" s="2">
-        <v>12.116333</v>
+        <v>10.746812</v>
       </c>
       <c r="J2" s="2">
         <v>12.116333</v>
       </c>
       <c r="K2" s="2">
-        <v>0.0</v>
+        <v>3.911968</v>
       </c>
       <c r="L2" s="2">
-        <v>12.116332</v>
+        <v>10.746811999999998</v>
       </c>
       <c r="M2" s="2">
         <v>0</v>
       </c>
       <c r="N2" s="3">
-        <v>45.978899999999996</v>
+        <v>41.82373333333333</v>
       </c>
       <c r="O2" s="3">
         <v>45.978899999999996</v>
       </c>
       <c r="P2" s="3">
-        <v>45.978899999999996</v>
+        <v>49.62625</v>
       </c>
       <c r="Q2" s="1">
         <v>18</v>
       </c>
       <c r="R2" s="1">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="S2" s="1">
         <v>5</v>
       </c>
       <c r="T2" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U2" s="1">
         <v>1</v>
@@ -51504,13 +51510,13 @@
         <v>0</v>
       </c>
       <c r="Z2" s="3">
-        <v>405.401</v>
+        <v>352.538</v>
       </c>
       <c r="AA2" s="3">
         <v>405.401</v>
       </c>
       <c r="AB2" s="3">
-        <v>371.552</v>
+        <v>279.836</v>
       </c>
       <c r="AC2" s="3">
         <v>371.552</v>
@@ -51524,40 +51530,40 @@
         <v>68</v>
       </c>
       <c r="C3" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" s="2">
-        <v>6.656134</v>
+        <v>6.249803333333333</v>
       </c>
       <c r="G3" s="2">
-        <v>6.656134</v>
+        <v>18.74941</v>
       </c>
       <c r="H3" s="2">
-        <v>6.656134</v>
+        <v>5.795459</v>
       </c>
       <c r="I3" s="2">
-        <v>6.656134</v>
+        <v>6.297817</v>
       </c>
       <c r="J3" s="2">
         <v>6.656134</v>
       </c>
       <c r="K3" s="2">
-        <v>0.0</v>
+        <v>0.8606749999999996</v>
       </c>
       <c r="L3" s="2">
-        <v>6.656134</v>
+        <v>6.297816</v>
       </c>
       <c r="M3" s="2">
         <v>0</v>
       </c>
       <c r="N3" s="3">
-        <v>44.932900000000004</v>
+        <v>40.727133333333335</v>
       </c>
       <c r="O3" s="3">
-        <v>44.932900000000004</v>
+        <v>43.91788333333333</v>
       </c>
       <c r="P3" s="3">
         <v>44.932900000000004</v>
@@ -51566,7 +51572,7 @@
         <v>4</v>
       </c>
       <c r="R3" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="S3" s="1">
         <v>3</v>
@@ -51593,10 +51599,10 @@
         <v>44.805</v>
       </c>
       <c r="AA3" s="3">
-        <v>44.805</v>
+        <v>60.352</v>
       </c>
       <c r="AB3" s="3">
-        <v>506.67</v>
+        <v>388.879</v>
       </c>
       <c r="AC3" s="3">
         <v>506.67</v>
@@ -51610,31 +51616,31 @@
         <v>80</v>
       </c>
       <c r="C4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="2">
-        <v>7.028553</v>
+        <v>7.779270333333333</v>
       </c>
       <c r="G4" s="2">
-        <v>7.028553</v>
+        <v>23.337811</v>
       </c>
       <c r="H4" s="2">
         <v>7.028553</v>
       </c>
       <c r="I4" s="2">
-        <v>7.028553</v>
+        <v>7.904781</v>
       </c>
       <c r="J4" s="2">
-        <v>7.028553</v>
+        <v>8.404477</v>
       </c>
       <c r="K4" s="2">
-        <v>0.0</v>
+        <v>1.3759240000000004</v>
       </c>
       <c r="L4" s="2">
-        <v>2.251192</v>
+        <v>3.100943</v>
       </c>
       <c r="M4" s="2">
         <v>4.777361</v>
@@ -51643,13 +51649,13 @@
         <v>47.0307</v>
       </c>
       <c r="O4" s="3">
-        <v>47.0307</v>
+        <v>53.20843333333333</v>
       </c>
       <c r="P4" s="3">
-        <v>47.0307</v>
+        <v>65.92375</v>
       </c>
       <c r="Q4" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="R4" s="1">
         <v>14</v>
@@ -51679,10 +51685,10 @@
         <v>111.026</v>
       </c>
       <c r="AA4" s="3">
-        <v>111.026</v>
+        <v>168.227</v>
       </c>
       <c r="AB4" s="3">
-        <v>186.027</v>
+        <v>131.067</v>
       </c>
       <c r="AC4" s="3">
         <v>186.027</v>
@@ -51696,52 +51702,52 @@
         <v>82</v>
       </c>
       <c r="C5" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D5" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" s="2">
-        <v>10.33528</v>
+        <v>11.217449</v>
       </c>
       <c r="G5" s="2">
-        <v>10.33528</v>
+        <v>33.652347</v>
       </c>
       <c r="H5" s="2">
         <v>10.33528</v>
       </c>
       <c r="I5" s="2">
-        <v>10.33528</v>
+        <v>10.422728</v>
       </c>
       <c r="J5" s="2">
-        <v>10.33528</v>
+        <v>12.894339</v>
       </c>
       <c r="K5" s="2">
-        <v>0.0</v>
+        <v>2.5590590000000013</v>
       </c>
       <c r="L5" s="2">
-        <v>8.729592</v>
+        <v>9.554582</v>
       </c>
       <c r="M5" s="2">
-        <v>1.605688</v>
+        <v>1.471124</v>
       </c>
       <c r="N5" s="3">
-        <v>41.971066666666665</v>
+        <v>31.6082</v>
       </c>
       <c r="O5" s="3">
         <v>41.971066666666665</v>
       </c>
       <c r="P5" s="3">
-        <v>41.971066666666665</v>
+        <v>46.82698333333334</v>
       </c>
       <c r="Q5" s="1">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="R5" s="1">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="S5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T5" s="1">
         <v>2</v>
@@ -51765,10 +51771,10 @@
         <v>294.098</v>
       </c>
       <c r="AA5" s="3">
-        <v>294.098</v>
+        <v>349.739</v>
       </c>
       <c r="AB5" s="3">
-        <v>126.892</v>
+        <v>111.622</v>
       </c>
       <c r="AC5" s="3">
         <v>126.892</v>
@@ -51783,7 +51789,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z60"/>
+  <dimension ref="A1:Z64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -54049,13 +54055,13 @@
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>787</v>
+        <v>110</v>
       </c>
       <c r="F30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30" t="b">
         <v>0</v>
@@ -54063,16 +54069,55 @@
       <c r="I30" s="4">
         <v>46315.22869212963</v>
       </c>
+      <c r="J30" s="4">
+        <v>46315.26194444444</v>
+      </c>
+      <c r="K30" s="3">
+        <v>41.82373333333333</v>
+      </c>
+      <c r="L30" s="2">
+        <v>8.204365</v>
+      </c>
+      <c r="M30" s="2">
+        <v>8.204365</v>
+      </c>
+      <c r="N30" s="2">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1">
+        <v>133</v>
+      </c>
+      <c r="P30" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q30" s="1">
+        <v>0</v>
+      </c>
+      <c r="R30" s="1">
+        <v>642.0</v>
+      </c>
+      <c r="S30" s="1">
+        <v>838704.0</v>
+      </c>
+      <c r="T30" s="1">
+        <v>50030478.0</v>
+      </c>
+      <c r="U30" s="1">
+        <v>1399751.0</v>
+      </c>
+      <c r="V30" s="1">
+        <v>352538</v>
+      </c>
+      <c r="W30" s="1">
+        <v>279836</v>
+      </c>
       <c r="X30" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y30" t="s">
-        <v>788</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B31" t="s">
         <v>61</v>
@@ -54096,137 +54141,134 @@
         <v>0</v>
       </c>
       <c r="I31" s="4">
-        <v>46314.29790509259</v>
+        <v>46315.258518518516</v>
       </c>
       <c r="J31" s="4">
-        <v>46314.32916666667</v>
+        <v>46315.2971875</v>
       </c>
       <c r="K31" s="3">
-        <v>39.51316666666666</v>
+        <v>49.62625</v>
       </c>
       <c r="L31" s="2">
-        <v>8.11915</v>
+        <v>10.746812</v>
       </c>
       <c r="M31" s="2">
-        <v>8.11915</v>
+        <v>10.746811999999998</v>
       </c>
       <c r="N31" s="2">
         <v>0</v>
       </c>
       <c r="O31" s="1">
-        <v>16</v>
+        <v>119</v>
       </c>
       <c r="P31" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q31" s="1">
         <v>0</v>
       </c>
       <c r="R31" s="1">
-        <v>666.0</v>
+        <v>868.0</v>
       </c>
       <c r="S31" s="1">
-        <v>710400.0</v>
+        <v>1026058.0</v>
       </c>
       <c r="T31" s="1">
-        <v>55968395.0</v>
+        <v>75790066.0</v>
       </c>
       <c r="U31" s="1">
-        <v>1169834.0</v>
+        <v>1735972.0</v>
       </c>
       <c r="V31" s="1">
-        <v>312594</v>
+        <v>364147</v>
       </c>
       <c r="W31" s="1">
-        <v>322948</v>
+        <v>314528</v>
       </c>
       <c r="X31" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y31" t="s">
-        <v>790</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C32" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D32" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E32" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" t="b">
         <v>0</v>
       </c>
       <c r="I32" s="4">
-        <v>46314.15864583333</v>
+        <v>46314.29790509259</v>
       </c>
       <c r="J32" s="4">
-        <v>46314.19634259259</v>
+        <v>46314.32916666667</v>
       </c>
       <c r="K32" s="3">
-        <v>48.41158333333333</v>
+        <v>39.51316666666666</v>
       </c>
       <c r="L32" s="2">
-        <v>8.756337</v>
+        <v>8.11915</v>
       </c>
       <c r="M32" s="2">
-        <v>8.756337</v>
+        <v>8.11915</v>
       </c>
       <c r="N32" s="2">
         <v>0</v>
       </c>
       <c r="O32" s="1">
-        <v>146</v>
+        <v>16</v>
       </c>
       <c r="P32" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q32" s="1">
         <v>0</v>
       </c>
       <c r="R32" s="1">
-        <v>282.0</v>
+        <v>666.0</v>
       </c>
       <c r="S32" s="1">
-        <v>279123.0</v>
+        <v>710400.0</v>
       </c>
       <c r="T32" s="1">
-        <v>40577429.0</v>
+        <v>55968395.0</v>
       </c>
       <c r="U32" s="1">
-        <v>476700.0</v>
+        <v>1169834.0</v>
       </c>
       <c r="V32" s="1">
-        <v>476702</v>
+        <v>312594</v>
+      </c>
+      <c r="W32" s="1">
+        <v>322948</v>
       </c>
       <c r="X32" t="b">
         <v>0</v>
       </c>
       <c r="Y32" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z32" t="s">
-        <v>751</v>
+        <v>789</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B33" t="s">
         <v>63</v>
@@ -54250,25 +54292,25 @@
         <v>0</v>
       </c>
       <c r="I33" s="4">
-        <v>46313.86145833333</v>
+        <v>46314.15864583333</v>
       </c>
       <c r="J33" s="4">
-        <v>46313.90385416667</v>
+        <v>46314.19634259259</v>
       </c>
       <c r="K33" s="3">
-        <v>54.91406666666667</v>
+        <v>48.41158333333333</v>
       </c>
       <c r="L33" s="2">
-        <v>10.22348</v>
+        <v>8.756337</v>
       </c>
       <c r="M33" s="2">
-        <v>10.22348</v>
+        <v>8.756337</v>
       </c>
       <c r="N33" s="2">
         <v>0</v>
       </c>
       <c r="O33" s="1">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="P33" s="1">
         <v>0</v>
@@ -54277,19 +54319,19 @@
         <v>0</v>
       </c>
       <c r="R33" s="1">
-        <v>320.0</v>
+        <v>282.0</v>
       </c>
       <c r="S33" s="1">
-        <v>299935.0</v>
+        <v>279123.0</v>
       </c>
       <c r="T33" s="1">
-        <v>51508661.0</v>
+        <v>40577429.0</v>
       </c>
       <c r="U33" s="1">
-        <v>518156.0</v>
+        <v>476700.0</v>
       </c>
       <c r="V33" s="1">
-        <v>523577</v>
+        <v>476702</v>
       </c>
       <c r="X33" t="b">
         <v>0</v>
@@ -54298,12 +54340,12 @@
         <v>432</v>
       </c>
       <c r="Z33" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="B34" t="s">
         <v>63</v>
@@ -54315,10 +54357,10 @@
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" s="1">
         <v>2</v>
@@ -54327,25 +54369,25 @@
         <v>0</v>
       </c>
       <c r="I34" s="4">
-        <v>46314.57332175926</v>
+        <v>46313.86145833333</v>
       </c>
       <c r="J34" s="4">
-        <v>46314.61576388889</v>
+        <v>46313.90385416667</v>
       </c>
       <c r="K34" s="3">
-        <v>50.72746666666667</v>
+        <v>54.91406666666667</v>
       </c>
       <c r="L34" s="2">
-        <v>11.371427</v>
+        <v>10.22348</v>
       </c>
       <c r="M34" s="2">
-        <v>11.371427</v>
+        <v>10.22348</v>
       </c>
       <c r="N34" s="2">
         <v>0</v>
       </c>
       <c r="O34" s="1">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="P34" s="1">
         <v>0</v>
@@ -54354,30 +54396,33 @@
         <v>0</v>
       </c>
       <c r="R34" s="1">
-        <v>352.0</v>
+        <v>320.0</v>
       </c>
       <c r="S34" s="1">
-        <v>323735.0</v>
+        <v>299935.0</v>
       </c>
       <c r="T34" s="1">
-        <v>58971088.0</v>
+        <v>51508661.0</v>
       </c>
       <c r="U34" s="1">
-        <v>559066.0</v>
+        <v>518156.0</v>
       </c>
       <c r="V34" s="1">
-        <v>559068</v>
+        <v>523577</v>
       </c>
       <c r="X34" t="b">
         <v>0</v>
       </c>
       <c r="Y34" t="s">
-        <v>794</v>
+        <v>432</v>
+      </c>
+      <c r="Z34" t="s">
+        <v>757</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="B35" t="s">
         <v>63</v>
@@ -54386,40 +54431,40 @@
         <v>64</v>
       </c>
       <c r="D35" s="1">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>110</v>
+      </c>
+      <c r="F35" t="b">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1">
         <v>2</v>
       </c>
-      <c r="E35" t="s">
-        <v>110</v>
-      </c>
-      <c r="F35" t="b">
-        <v>1</v>
-      </c>
-      <c r="G35" s="1">
-        <v>1</v>
-      </c>
       <c r="H35" t="b">
         <v>0</v>
       </c>
       <c r="I35" s="4">
-        <v>46314.160046296296</v>
+        <v>46314.57332175926</v>
       </c>
       <c r="J35" s="4">
-        <v>46314.19709490741</v>
+        <v>46314.61576388889</v>
       </c>
       <c r="K35" s="3">
-        <v>48.04756666666666</v>
+        <v>50.72746666666667</v>
       </c>
       <c r="L35" s="2">
-        <v>9.165487</v>
+        <v>11.371427</v>
       </c>
       <c r="M35" s="2">
-        <v>9.165487</v>
+        <v>11.371427</v>
       </c>
       <c r="N35" s="2">
         <v>0</v>
       </c>
       <c r="O35" s="1">
-        <v>150</v>
+        <v>178</v>
       </c>
       <c r="P35" s="1">
         <v>0</v>
@@ -54428,30 +54473,30 @@
         <v>0</v>
       </c>
       <c r="R35" s="1">
-        <v>294.0</v>
+        <v>352.0</v>
       </c>
       <c r="S35" s="1">
-        <v>289718.0</v>
+        <v>323735.0</v>
       </c>
       <c r="T35" s="1">
-        <v>42949072.0</v>
+        <v>58971088.0</v>
       </c>
       <c r="U35" s="1">
-        <v>493203.0</v>
+        <v>559066.0</v>
       </c>
       <c r="V35" s="1">
-        <v>498624</v>
+        <v>559068</v>
       </c>
       <c r="X35" t="b">
         <v>0</v>
       </c>
       <c r="Y35" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="B36" t="s">
         <v>63</v>
@@ -54460,40 +54505,40 @@
         <v>64</v>
       </c>
       <c r="D36" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36" t="s">
         <v>110</v>
       </c>
       <c r="F36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36" s="4">
-        <v>46314.32548611111</v>
+        <v>46314.160046296296</v>
       </c>
       <c r="J36" s="4">
-        <v>46314.41706018519</v>
+        <v>46314.19709490741</v>
       </c>
       <c r="K36" s="3">
-        <v>104.91581666666666</v>
+        <v>48.04756666666666</v>
       </c>
       <c r="L36" s="2">
-        <v>21.168002</v>
+        <v>9.165487</v>
       </c>
       <c r="M36" s="2">
-        <v>21.168002</v>
+        <v>9.165487</v>
       </c>
       <c r="N36" s="2">
         <v>0</v>
       </c>
       <c r="O36" s="1">
-        <v>98</v>
+        <v>150</v>
       </c>
       <c r="P36" s="1">
         <v>0</v>
@@ -54502,42 +54547,42 @@
         <v>0</v>
       </c>
       <c r="R36" s="1">
-        <v>582.0</v>
+        <v>294.0</v>
       </c>
       <c r="S36" s="1">
-        <v>498236.0</v>
+        <v>289718.0</v>
       </c>
       <c r="T36" s="1">
-        <v>131478461.0</v>
+        <v>42949072.0</v>
       </c>
       <c r="U36" s="1">
-        <v>759158.0</v>
+        <v>493203.0</v>
       </c>
       <c r="V36" s="1">
-        <v>764579</v>
+        <v>498624</v>
       </c>
       <c r="X36" t="b">
         <v>0</v>
       </c>
       <c r="Y36" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="B37" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D37" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E37" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
@@ -54546,66 +54591,60 @@
         <v>5</v>
       </c>
       <c r="H37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="4">
-        <v>46313.86164351852</v>
+        <v>46314.32548611111</v>
       </c>
       <c r="J37" s="4">
-        <v>46313.90555555555</v>
+        <v>46314.41706018519</v>
       </c>
       <c r="K37" s="3">
-        <v>51.99661666666667</v>
+        <v>104.91581666666666</v>
       </c>
       <c r="L37" s="2">
-        <v>7.706352</v>
+        <v>21.168002</v>
       </c>
       <c r="M37" s="2">
-        <v>7.706352</v>
+        <v>21.168002</v>
       </c>
       <c r="N37" s="2">
         <v>0</v>
       </c>
       <c r="O37" s="1">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="P37" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="Q37" s="1">
         <v>0</v>
       </c>
       <c r="R37" s="1">
-        <v>924.0</v>
+        <v>582.0</v>
       </c>
       <c r="S37" s="1">
-        <v>779272.0</v>
+        <v>498236.0</v>
       </c>
       <c r="T37" s="1">
-        <v>48456621.0</v>
+        <v>131478461.0</v>
       </c>
       <c r="U37" s="1">
-        <v>1705620.0</v>
+        <v>759158.0</v>
       </c>
       <c r="V37" s="1">
-        <v>85496</v>
-      </c>
-      <c r="W37" s="1">
-        <v>257260</v>
+        <v>764579</v>
       </c>
       <c r="X37" t="b">
         <v>0</v>
       </c>
       <c r="Y37" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z37" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="B38" t="s">
         <v>67</v>
@@ -54617,69 +54656,75 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H38" t="b">
         <v>0</v>
       </c>
       <c r="I38" s="4">
-        <v>46315.19493055555</v>
+        <v>46313.86164351852</v>
       </c>
       <c r="J38" s="4">
-        <v>46315.23050925926</v>
+        <v>46313.90555555555</v>
       </c>
       <c r="K38" s="3">
-        <v>44.932900000000004</v>
+        <v>51.99661666666667</v>
       </c>
       <c r="L38" s="2">
-        <v>6.656134</v>
+        <v>7.706352</v>
       </c>
       <c r="M38" s="2">
-        <v>6.656134</v>
+        <v>7.706352</v>
       </c>
       <c r="N38" s="2">
         <v>0</v>
       </c>
       <c r="O38" s="1">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="P38" s="1">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="Q38" s="1">
         <v>0</v>
       </c>
       <c r="R38" s="1">
-        <v>460.0</v>
+        <v>924.0</v>
       </c>
       <c r="S38" s="1">
-        <v>509481.0</v>
+        <v>779272.0</v>
       </c>
       <c r="T38" s="1">
-        <v>44845086.0</v>
+        <v>48456621.0</v>
       </c>
       <c r="U38" s="1">
-        <v>861558.0</v>
+        <v>1705620.0</v>
       </c>
       <c r="V38" s="1">
-        <v>44805</v>
+        <v>85496</v>
       </c>
       <c r="W38" s="1">
-        <v>506670</v>
+        <v>257260</v>
       </c>
       <c r="X38" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>432</v>
+      </c>
+      <c r="Z38" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="B39" t="s">
         <v>67</v>
@@ -54697,66 +54742,63 @@
         <v>1</v>
       </c>
       <c r="G39" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H39" t="b">
         <v>0</v>
       </c>
       <c r="I39" s="4">
-        <v>46314.584178240744</v>
+        <v>46315.19493055555</v>
       </c>
       <c r="J39" s="4">
-        <v>46314.63313657408</v>
+        <v>46315.23050925926</v>
       </c>
       <c r="K39" s="3">
-        <v>60.036500000000004</v>
+        <v>44.932900000000004</v>
       </c>
       <c r="L39" s="2">
-        <v>5.548321</v>
+        <v>6.656134</v>
       </c>
       <c r="M39" s="2">
-        <v>5.548322</v>
+        <v>6.656134</v>
       </c>
       <c r="N39" s="2">
         <v>0</v>
       </c>
       <c r="O39" s="1">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="P39" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q39" s="1">
         <v>0</v>
       </c>
       <c r="R39" s="1">
-        <v>520.0</v>
+        <v>460.0</v>
       </c>
       <c r="S39" s="1">
-        <v>539478.0</v>
+        <v>509481.0</v>
       </c>
       <c r="T39" s="1">
-        <v>36078318.0</v>
+        <v>44845086.0</v>
       </c>
       <c r="U39" s="1">
-        <v>948571.0</v>
+        <v>861558.0</v>
       </c>
       <c r="V39" s="1">
-        <v>48307</v>
+        <v>44805</v>
       </c>
       <c r="W39" s="1">
-        <v>380955</v>
+        <v>506670</v>
       </c>
       <c r="X39" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y39" t="s">
-        <v>803</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B40" t="s">
         <v>67</v>
@@ -54768,10 +54810,10 @@
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="1">
         <v>2</v>
@@ -54780,25 +54822,25 @@
         <v>0</v>
       </c>
       <c r="I40" s="4">
-        <v>46314.15881944444</v>
+        <v>46314.584178240744</v>
       </c>
       <c r="J40" s="4">
-        <v>46314.19364583334</v>
+        <v>46314.63313657408</v>
       </c>
       <c r="K40" s="3">
-        <v>44.1155</v>
+        <v>60.036500000000004</v>
       </c>
       <c r="L40" s="2">
-        <v>3.875124</v>
+        <v>5.548321</v>
       </c>
       <c r="M40" s="2">
-        <v>3.875124</v>
+        <v>5.548322</v>
       </c>
       <c r="N40" s="2">
         <v>0</v>
       </c>
       <c r="O40" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P40" s="1">
         <v>4</v>
@@ -54807,36 +54849,33 @@
         <v>0</v>
       </c>
       <c r="R40" s="1">
-        <v>540.0</v>
+        <v>520.0</v>
       </c>
       <c r="S40" s="1">
-        <v>529894.0</v>
+        <v>539478.0</v>
       </c>
       <c r="T40" s="1">
-        <v>35974215.0</v>
+        <v>36078318.0</v>
       </c>
       <c r="U40" s="1">
-        <v>997521.0</v>
+        <v>948571.0</v>
       </c>
       <c r="V40" s="1">
-        <v>47980</v>
+        <v>48307</v>
       </c>
       <c r="W40" s="1">
-        <v>293478</v>
+        <v>380955</v>
       </c>
       <c r="X40" t="b">
         <v>0</v>
       </c>
       <c r="Y40" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z40" t="s">
-        <v>751</v>
+        <v>802</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="B41" t="s">
         <v>67</v>
@@ -54845,13 +54884,13 @@
         <v>68</v>
       </c>
       <c r="D41" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" s="1">
         <v>2</v>
@@ -54860,25 +54899,25 @@
         <v>0</v>
       </c>
       <c r="I41" s="4">
-        <v>46314.210381944446</v>
+        <v>46314.15881944444</v>
       </c>
       <c r="J41" s="4">
-        <v>46314.25950231482</v>
+        <v>46314.19364583334</v>
       </c>
       <c r="K41" s="3">
-        <v>59.42836666666667</v>
+        <v>44.1155</v>
       </c>
       <c r="L41" s="2">
-        <v>8.398512</v>
+        <v>3.875124</v>
       </c>
       <c r="M41" s="2">
-        <v>8.398512</v>
+        <v>3.875124</v>
       </c>
       <c r="N41" s="2">
         <v>0</v>
       </c>
       <c r="O41" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="P41" s="1">
         <v>4</v>
@@ -54887,33 +54926,36 @@
         <v>0</v>
       </c>
       <c r="R41" s="1">
-        <v>618.0</v>
+        <v>540.0</v>
       </c>
       <c r="S41" s="1">
-        <v>621706.0</v>
+        <v>529894.0</v>
       </c>
       <c r="T41" s="1">
-        <v>54903298.0</v>
+        <v>35974215.0</v>
       </c>
       <c r="U41" s="1">
-        <v>1155513.0</v>
+        <v>997521.0</v>
       </c>
       <c r="V41" s="1">
-        <v>64109</v>
+        <v>47980</v>
       </c>
       <c r="W41" s="1">
-        <v>427464</v>
+        <v>293478</v>
       </c>
       <c r="X41" t="b">
         <v>0</v>
       </c>
       <c r="Y41" t="s">
-        <v>806</v>
+        <v>432</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="B42" t="s">
         <v>67</v>
@@ -54925,30 +54967,72 @@
         <v>2</v>
       </c>
       <c r="E42" t="s">
-        <v>787</v>
+        <v>110</v>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H42" t="b">
         <v>0</v>
       </c>
       <c r="I42" s="4">
-        <v>46315.230729166666</v>
+        <v>46314.210381944446</v>
+      </c>
+      <c r="J42" s="4">
+        <v>46314.25950231482</v>
+      </c>
+      <c r="K42" s="3">
+        <v>59.42836666666667</v>
+      </c>
+      <c r="L42" s="2">
+        <v>8.398512</v>
+      </c>
+      <c r="M42" s="2">
+        <v>8.398512</v>
+      </c>
+      <c r="N42" s="2">
+        <v>0</v>
+      </c>
+      <c r="O42" s="1">
+        <v>10</v>
+      </c>
+      <c r="P42" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q42" s="1">
+        <v>0</v>
+      </c>
+      <c r="R42" s="1">
+        <v>618.0</v>
+      </c>
+      <c r="S42" s="1">
+        <v>621706.0</v>
+      </c>
+      <c r="T42" s="1">
+        <v>54903298.0</v>
+      </c>
+      <c r="U42" s="1">
+        <v>1155513.0</v>
+      </c>
+      <c r="V42" s="1">
+        <v>64109</v>
+      </c>
+      <c r="W42" s="1">
+        <v>427464</v>
       </c>
       <c r="X42" t="b">
         <v>0</v>
       </c>
       <c r="Y42" t="s">
-        <v>788</v>
+        <v>805</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="B43" t="s">
         <v>67</v>
@@ -54957,235 +55041,223 @@
         <v>68</v>
       </c>
       <c r="D43" s="1">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+      <c r="G43" s="1">
+        <v>1</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4">
+        <v>46315.230729166666</v>
+      </c>
+      <c r="J43" s="4">
+        <v>46315.26327546296</v>
+      </c>
+      <c r="K43" s="3">
+        <v>40.727133333333335</v>
+      </c>
+      <c r="L43" s="2">
+        <v>5.795459</v>
+      </c>
+      <c r="M43" s="2">
+        <v>5.795459</v>
+      </c>
+      <c r="N43" s="2">
+        <v>0</v>
+      </c>
+      <c r="O43" s="1">
+        <v>5</v>
+      </c>
+      <c r="P43" s="1">
         <v>3</v>
       </c>
-      <c r="E43" t="s">
-        <v>110</v>
-      </c>
-      <c r="F43" t="b">
-        <v>1</v>
-      </c>
-      <c r="G43" s="1">
-        <v>3</v>
-      </c>
-      <c r="H43" t="b">
-        <v>0</v>
-      </c>
-      <c r="I43" s="4">
-        <v>46314.32938657407</v>
-      </c>
-      <c r="J43" s="4">
-        <v>46314.379849537036</v>
-      </c>
-      <c r="K43" s="3">
-        <v>55.412016666666666</v>
-      </c>
-      <c r="L43" s="2">
-        <v>8.53418</v>
-      </c>
-      <c r="M43" s="2">
-        <v>8.53418</v>
-      </c>
-      <c r="N43" s="2">
-        <v>0</v>
-      </c>
-      <c r="O43" s="1">
-        <v>32</v>
-      </c>
-      <c r="P43" s="1">
-        <v>7</v>
-      </c>
       <c r="Q43" s="1">
         <v>0</v>
       </c>
       <c r="R43" s="1">
-        <v>834.0</v>
+        <v>404.0</v>
       </c>
       <c r="S43" s="1">
-        <v>839688.0</v>
+        <v>446176.0</v>
       </c>
       <c r="T43" s="1">
-        <v>54499916.0</v>
+        <v>32379531.0</v>
       </c>
       <c r="U43" s="1">
-        <v>1684516.0</v>
+        <v>791519.0</v>
       </c>
       <c r="V43" s="1">
-        <v>81975</v>
+        <v>52413</v>
       </c>
       <c r="W43" s="1">
-        <v>299031</v>
+        <v>435672</v>
       </c>
       <c r="X43" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y43" t="s">
-        <v>809</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B44" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D44" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" s="1">
+        <v>1</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" s="4">
+        <v>46315.2621875</v>
+      </c>
+      <c r="J44" s="4">
+        <v>46315.296944444446</v>
+      </c>
+      <c r="K44" s="3">
+        <v>43.91788333333333</v>
+      </c>
+      <c r="L44" s="2">
+        <v>6.297817</v>
+      </c>
+      <c r="M44" s="2">
+        <v>6.297816</v>
+      </c>
+      <c r="N44" s="2">
+        <v>0</v>
+      </c>
+      <c r="O44" s="1">
+        <v>8</v>
+      </c>
+      <c r="P44" s="1">
         <v>3</v>
       </c>
-      <c r="H44" t="b">
-        <v>0</v>
-      </c>
-      <c r="I44" s="4">
-        <v>46314.15899305556</v>
-      </c>
-      <c r="J44" s="4">
-        <v>46314.193460648145</v>
-      </c>
-      <c r="K44" s="3">
-        <v>49.385549999999995</v>
-      </c>
-      <c r="L44" s="2">
-        <v>10.350417</v>
-      </c>
-      <c r="M44" s="2">
-        <v>10.350418</v>
-      </c>
-      <c r="N44" s="2">
-        <v>0</v>
-      </c>
-      <c r="O44" s="1">
-        <v>37</v>
-      </c>
-      <c r="P44" s="1">
-        <v>7</v>
-      </c>
       <c r="Q44" s="1">
         <v>0</v>
       </c>
       <c r="R44" s="1">
-        <v>1084.0</v>
+        <v>474.0</v>
       </c>
       <c r="S44" s="1">
-        <v>986438.0</v>
+        <v>423579.0</v>
       </c>
       <c r="T44" s="1">
-        <v>88431683.0</v>
+        <v>33008177.0</v>
       </c>
       <c r="U44" s="1">
-        <v>1905956.0</v>
+        <v>797744.0</v>
       </c>
       <c r="V44" s="1">
-        <v>236869</v>
+        <v>60352</v>
       </c>
       <c r="W44" s="1">
-        <v>376179</v>
+        <v>388879</v>
       </c>
       <c r="X44" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y44" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z44" t="s">
-        <v>811</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
       <c r="B45" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C45" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D45" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E45" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H45" t="b">
         <v>0</v>
       </c>
       <c r="I45" s="4">
-        <v>46313.862280092595</v>
+        <v>46314.32938657407</v>
       </c>
       <c r="J45" s="4">
-        <v>46313.90387731481</v>
+        <v>46314.379849537036</v>
       </c>
       <c r="K45" s="3">
-        <v>54.19301666666667</v>
+        <v>55.412016666666666</v>
       </c>
       <c r="L45" s="2">
-        <v>11.580787</v>
+        <v>8.53418</v>
       </c>
       <c r="M45" s="2">
-        <v>11.580788</v>
+        <v>8.53418</v>
       </c>
       <c r="N45" s="2">
         <v>0</v>
       </c>
       <c r="O45" s="1">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="P45" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q45" s="1">
         <v>0</v>
       </c>
       <c r="R45" s="1">
-        <v>576.0</v>
+        <v>834.0</v>
       </c>
       <c r="S45" s="1">
-        <v>486536.0</v>
+        <v>839688.0</v>
       </c>
       <c r="T45" s="1">
-        <v>43600123.0</v>
+        <v>54499916.0</v>
       </c>
       <c r="U45" s="1">
-        <v>1090895.0</v>
+        <v>1684516.0</v>
       </c>
       <c r="V45" s="1">
-        <v>157439</v>
+        <v>81975</v>
       </c>
       <c r="W45" s="1">
-        <v>369085</v>
+        <v>299031</v>
       </c>
       <c r="X45" t="b">
         <v>0</v>
       </c>
       <c r="Y45" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z45" t="s">
-        <v>757</v>
+        <v>809</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="B46" t="s">
         <v>69</v>
@@ -55197,72 +55269,75 @@
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H46" t="b">
         <v>0</v>
       </c>
       <c r="I46" s="4">
-        <v>46314.586909722224</v>
+        <v>46314.15899305556</v>
       </c>
       <c r="J46" s="4">
-        <v>46314.640069444446</v>
+        <v>46314.193460648145</v>
       </c>
       <c r="K46" s="3">
-        <v>65.17911666666666</v>
+        <v>49.385549999999995</v>
       </c>
       <c r="L46" s="2">
-        <v>10.446109</v>
+        <v>10.350417</v>
       </c>
       <c r="M46" s="2">
-        <v>10.446109</v>
+        <v>10.350418</v>
       </c>
       <c r="N46" s="2">
         <v>0</v>
       </c>
       <c r="O46" s="1">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="P46" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q46" s="1">
         <v>0</v>
       </c>
       <c r="R46" s="1">
-        <v>722.0</v>
+        <v>1084.0</v>
       </c>
       <c r="S46" s="1">
-        <v>708289.0</v>
+        <v>986438.0</v>
       </c>
       <c r="T46" s="1">
-        <v>51642018.0</v>
+        <v>88431683.0</v>
       </c>
       <c r="U46" s="1">
-        <v>1305105.0</v>
+        <v>1905956.0</v>
       </c>
       <c r="V46" s="1">
-        <v>179932</v>
+        <v>236869</v>
       </c>
       <c r="W46" s="1">
-        <v>420234</v>
+        <v>376179</v>
       </c>
       <c r="X46" t="b">
         <v>0</v>
       </c>
       <c r="Y46" t="s">
-        <v>814</v>
+        <v>432</v>
+      </c>
+      <c r="Z46" t="s">
+        <v>811</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="B47" t="s">
         <v>69</v>
@@ -55271,75 +55346,78 @@
         <v>70</v>
       </c>
       <c r="D47" s="1">
+        <v>1</v>
+      </c>
+      <c r="E47" t="s">
+        <v>431</v>
+      </c>
+      <c r="F47" t="b">
+        <v>0</v>
+      </c>
+      <c r="G47" s="1">
         <v>2</v>
       </c>
-      <c r="E47" t="s">
-        <v>110</v>
-      </c>
-      <c r="F47" t="b">
-        <v>1</v>
-      </c>
-      <c r="G47" s="1">
-        <v>3</v>
-      </c>
       <c r="H47" t="b">
         <v>0</v>
       </c>
       <c r="I47" s="4">
-        <v>46314.21055555555</v>
+        <v>46313.862280092595</v>
       </c>
       <c r="J47" s="4">
-        <v>46314.25184027778</v>
+        <v>46313.90387731481</v>
       </c>
       <c r="K47" s="3">
-        <v>48.78155</v>
+        <v>54.19301666666667</v>
       </c>
       <c r="L47" s="2">
-        <v>12.718512</v>
+        <v>11.580787</v>
       </c>
       <c r="M47" s="2">
-        <v>12.718512</v>
+        <v>11.580788</v>
       </c>
       <c r="N47" s="2">
         <v>0</v>
       </c>
       <c r="O47" s="1">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="P47" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q47" s="1">
         <v>0</v>
       </c>
       <c r="R47" s="1">
-        <v>882.0</v>
+        <v>576.0</v>
       </c>
       <c r="S47" s="1">
-        <v>945280.0</v>
+        <v>486536.0</v>
       </c>
       <c r="T47" s="1">
-        <v>64072835.0</v>
+        <v>43600123.0</v>
       </c>
       <c r="U47" s="1">
-        <v>1711070.0</v>
+        <v>1090895.0</v>
       </c>
       <c r="V47" s="1">
-        <v>223412</v>
+        <v>157439</v>
       </c>
       <c r="W47" s="1">
-        <v>358765</v>
+        <v>369085</v>
       </c>
       <c r="X47" t="b">
         <v>0</v>
       </c>
       <c r="Y47" t="s">
-        <v>816</v>
+        <v>432</v>
+      </c>
+      <c r="Z47" t="s">
+        <v>757</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
       <c r="B48" t="s">
         <v>69</v>
@@ -55348,7 +55426,7 @@
         <v>70</v>
       </c>
       <c r="D48" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E48" t="s">
         <v>110</v>
@@ -55363,69 +55441,69 @@
         <v>0</v>
       </c>
       <c r="I48" s="4">
-        <v>46314.33002314815</v>
+        <v>46314.586909722224</v>
       </c>
       <c r="J48" s="4">
-        <v>46314.3778125</v>
+        <v>46314.640069444446</v>
       </c>
       <c r="K48" s="3">
-        <v>58.06751666666666</v>
+        <v>65.17911666666666</v>
       </c>
       <c r="L48" s="2">
-        <v>9.519687</v>
+        <v>10.446109</v>
       </c>
       <c r="M48" s="2">
-        <v>9.519686</v>
+        <v>10.446109</v>
       </c>
       <c r="N48" s="2">
         <v>0</v>
       </c>
       <c r="O48" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="P48" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q48" s="1">
         <v>0</v>
       </c>
       <c r="R48" s="1">
-        <v>528.0</v>
+        <v>722.0</v>
       </c>
       <c r="S48" s="1">
-        <v>564432.0</v>
+        <v>708289.0</v>
       </c>
       <c r="T48" s="1">
-        <v>41322323.0</v>
+        <v>51642018.0</v>
       </c>
       <c r="U48" s="1">
-        <v>971256.0</v>
+        <v>1305105.0</v>
       </c>
       <c r="V48" s="1">
-        <v>132839</v>
+        <v>179932</v>
       </c>
       <c r="W48" s="1">
-        <v>445527</v>
+        <v>420234</v>
       </c>
       <c r="X48" t="b">
         <v>0</v>
       </c>
       <c r="Y48" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="B49" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D49" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="s">
         <v>110</v>
@@ -55440,72 +55518,75 @@
         <v>0</v>
       </c>
       <c r="I49" s="4">
-        <v>46314.59266203704</v>
+        <v>46314.21055555555</v>
       </c>
       <c r="J49" s="4">
-        <v>46314.654490740744</v>
+        <v>46314.25184027778</v>
       </c>
       <c r="K49" s="3">
-        <v>73.2598</v>
+        <v>48.78155</v>
       </c>
       <c r="L49" s="2">
-        <v>9.924175</v>
+        <v>12.718512</v>
       </c>
       <c r="M49" s="2">
-        <v>9.924175</v>
+        <v>12.718512</v>
       </c>
       <c r="N49" s="2">
         <v>0</v>
       </c>
       <c r="O49" s="1">
-        <v>293</v>
+        <v>51</v>
       </c>
       <c r="P49" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q49" s="1">
         <v>0</v>
       </c>
       <c r="R49" s="1">
-        <v>582.0</v>
+        <v>882.0</v>
       </c>
       <c r="S49" s="1">
-        <v>644532.0</v>
+        <v>945280.0</v>
       </c>
       <c r="T49" s="1">
-        <v>151776389.0</v>
+        <v>64072835.0</v>
       </c>
       <c r="U49" s="1">
-        <v>884968.0</v>
+        <v>1711070.0</v>
       </c>
       <c r="V49" s="1">
-        <v>884970</v>
+        <v>223412</v>
+      </c>
+      <c r="W49" s="1">
+        <v>358765</v>
       </c>
       <c r="X49" t="b">
         <v>0</v>
       </c>
       <c r="Y49" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="B50" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C50" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D50" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E50" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="1">
         <v>2</v>
@@ -55514,60 +55595,60 @@
         <v>0</v>
       </c>
       <c r="I50" s="4">
-        <v>46314.159166666665</v>
+        <v>46314.33002314815</v>
       </c>
       <c r="J50" s="4">
-        <v>46314.19351851852</v>
+        <v>46314.3778125</v>
       </c>
       <c r="K50" s="3">
-        <v>43.80995</v>
+        <v>58.06751666666666</v>
       </c>
       <c r="L50" s="2">
-        <v>1.351832</v>
+        <v>9.519687</v>
       </c>
       <c r="M50" s="2">
-        <v>1.351832</v>
+        <v>9.519686</v>
       </c>
       <c r="N50" s="2">
         <v>0</v>
       </c>
       <c r="O50" s="1">
-        <v>235</v>
+        <v>33</v>
       </c>
       <c r="P50" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q50" s="1">
         <v>0</v>
       </c>
       <c r="R50" s="1">
-        <v>432.0</v>
+        <v>528.0</v>
       </c>
       <c r="S50" s="1">
-        <v>538506.0</v>
+        <v>564432.0</v>
       </c>
       <c r="T50" s="1">
-        <v>92764505.0</v>
+        <v>41322323.0</v>
       </c>
       <c r="U50" s="1">
-        <v>774455.0</v>
+        <v>971256.0</v>
       </c>
       <c r="V50" s="1">
-        <v>779876</v>
+        <v>132839</v>
+      </c>
+      <c r="W50" s="1">
+        <v>445527</v>
       </c>
       <c r="X50" t="b">
         <v>0</v>
       </c>
       <c r="Y50" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z50" t="s">
-        <v>751</v>
+        <v>818</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="B51" t="s">
         <v>71</v>
@@ -55576,72 +55657,72 @@
         <v>72</v>
       </c>
       <c r="D51" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" t="s">
         <v>110</v>
       </c>
       <c r="F51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G51" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I51" s="4">
-        <v>46314.21072916667</v>
+        <v>46314.59266203704</v>
       </c>
       <c r="J51" s="4">
-        <v>46314.29785879629</v>
+        <v>46314.654490740744</v>
       </c>
       <c r="K51" s="3">
-        <v>99.19116666666667</v>
+        <v>73.2598</v>
       </c>
       <c r="L51" s="2">
-        <v>14.433891</v>
+        <v>9.924175</v>
       </c>
       <c r="M51" s="2">
-        <v>14.433891</v>
+        <v>9.924175</v>
       </c>
       <c r="N51" s="2">
         <v>0</v>
       </c>
       <c r="O51" s="1">
-        <v>182</v>
+        <v>293</v>
       </c>
       <c r="P51" s="1">
         <v>0</v>
       </c>
       <c r="Q51" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R51" s="1">
-        <v>944.0</v>
+        <v>582.0</v>
       </c>
       <c r="S51" s="1">
-        <v>719044.0</v>
+        <v>644532.0</v>
       </c>
       <c r="T51" s="1">
-        <v>235843525.0</v>
+        <v>151776389.0</v>
       </c>
       <c r="U51" s="1">
-        <v>1151474.0</v>
+        <v>884968.0</v>
       </c>
       <c r="V51" s="1">
-        <v>963737</v>
+        <v>884970</v>
       </c>
       <c r="X51" t="b">
         <v>0</v>
       </c>
       <c r="Y51" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="B52" t="s">
         <v>71</v>
@@ -55650,190 +55731,223 @@
         <v>72</v>
       </c>
       <c r="D52" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F52" t="b">
         <v>0</v>
       </c>
       <c r="G52" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I52" s="4">
-        <v>46314.354363425926</v>
+        <v>46314.159166666665</v>
       </c>
       <c r="J52" s="4">
-        <v>46314.44310185185</v>
+        <v>46314.19351851852</v>
       </c>
       <c r="K52" s="3">
-        <v>100.32289999999999</v>
+        <v>43.80995</v>
       </c>
       <c r="L52" s="2">
-        <v>13.363789</v>
+        <v>1.351832</v>
       </c>
       <c r="M52" s="2">
-        <v>13.363789</v>
+        <v>1.351832</v>
       </c>
       <c r="N52" s="2">
         <v>0</v>
       </c>
       <c r="O52" s="1">
-        <v>478</v>
+        <v>235</v>
       </c>
       <c r="P52" s="1">
         <v>0</v>
       </c>
       <c r="Q52" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R52" s="1">
-        <v>954.0</v>
+        <v>432.0</v>
       </c>
       <c r="S52" s="1">
-        <v>905505.0</v>
+        <v>538506.0</v>
       </c>
       <c r="T52" s="1">
-        <v>202004019.0</v>
+        <v>92764505.0</v>
       </c>
       <c r="U52" s="1">
-        <v>1311783.0</v>
+        <v>774455.0</v>
       </c>
       <c r="V52" s="1">
-        <v>965871</v>
+        <v>779876</v>
       </c>
       <c r="X52" t="b">
         <v>0</v>
       </c>
       <c r="Y52" t="s">
-        <v>825</v>
+        <v>432</v>
+      </c>
+      <c r="Z52" t="s">
+        <v>751</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="B53" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C53" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D53" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E53" t="s">
-        <v>431</v>
+        <v>110</v>
       </c>
       <c r="F53" t="b">
         <v>0</v>
       </c>
       <c r="G53" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" s="4">
-        <v>46314.15934027778</v>
+        <v>46314.21072916667</v>
       </c>
       <c r="J53" s="4">
-        <v>46314.193449074075</v>
+        <v>46314.29785879629</v>
       </c>
       <c r="K53" s="3">
-        <v>49.05461666666667</v>
+        <v>99.19116666666667</v>
       </c>
       <c r="L53" s="2">
-        <v>1.393549</v>
+        <v>14.433891</v>
       </c>
       <c r="M53" s="2">
-        <v>1.393549</v>
+        <v>14.433891</v>
       </c>
       <c r="N53" s="2">
         <v>0</v>
       </c>
       <c r="O53" s="1">
-        <v>218</v>
+        <v>182</v>
       </c>
       <c r="P53" s="1">
         <v>0</v>
       </c>
       <c r="Q53" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R53" s="1">
-        <v>432.0</v>
+        <v>944.0</v>
       </c>
       <c r="S53" s="1">
-        <v>554729.0</v>
+        <v>719044.0</v>
       </c>
       <c r="T53" s="1">
-        <v>96089496.0</v>
+        <v>235843525.0</v>
       </c>
       <c r="U53" s="1">
-        <v>776230.0</v>
+        <v>1151474.0</v>
       </c>
       <c r="V53" s="1">
-        <v>781651</v>
+        <v>963737</v>
       </c>
       <c r="X53" t="b">
         <v>0</v>
       </c>
       <c r="Y53" t="s">
-        <v>432</v>
-      </c>
-      <c r="Z53" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>828</v>
+        <v>824</v>
       </c>
       <c r="B54" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C54" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D54" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E54" t="s">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="F54" t="b">
         <v>0</v>
       </c>
       <c r="G54" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" s="4">
-        <v>46314.69179398148</v>
+        <v>46314.354363425926</v>
       </c>
       <c r="J54" s="4">
-        <v>46314.70092592593</v>
+        <v>46314.44310185185</v>
+      </c>
+      <c r="K54" s="3">
+        <v>100.32289999999999</v>
+      </c>
+      <c r="L54" s="2">
+        <v>13.363789</v>
+      </c>
+      <c r="M54" s="2">
+        <v>13.363789</v>
+      </c>
+      <c r="N54" s="2">
+        <v>0</v>
+      </c>
+      <c r="O54" s="1">
+        <v>478</v>
+      </c>
+      <c r="P54" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="1">
+        <v>1</v>
+      </c>
+      <c r="R54" s="1">
+        <v>954.0</v>
+      </c>
+      <c r="S54" s="1">
+        <v>905505.0</v>
+      </c>
+      <c r="T54" s="1">
+        <v>202004019.0</v>
+      </c>
+      <c r="U54" s="1">
+        <v>1311783.0</v>
+      </c>
+      <c r="V54" s="1">
+        <v>965871</v>
       </c>
       <c r="X54" t="b">
         <v>0</v>
       </c>
       <c r="Y54" t="s">
-        <v>196</v>
-      </c>
-      <c r="Z54" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="B55" t="s">
         <v>73</v>
@@ -55842,72 +55956,75 @@
         <v>74</v>
       </c>
       <c r="D55" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" t="s">
-        <v>110</v>
+        <v>431</v>
       </c>
       <c r="F55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H55" t="b">
         <v>0</v>
       </c>
       <c r="I55" s="4">
-        <v>46314.25201388889</v>
+        <v>46314.15934027778</v>
       </c>
       <c r="J55" s="4">
-        <v>46314.32546296297</v>
+        <v>46314.193449074075</v>
       </c>
       <c r="K55" s="3">
-        <v>95.18496666666667</v>
+        <v>49.05461666666667</v>
       </c>
       <c r="L55" s="2">
-        <v>10.606161</v>
+        <v>1.393549</v>
       </c>
       <c r="M55" s="2">
-        <v>10.606161</v>
+        <v>1.393549</v>
       </c>
       <c r="N55" s="2">
         <v>0</v>
       </c>
       <c r="O55" s="1">
-        <v>335</v>
+        <v>218</v>
       </c>
       <c r="P55" s="1">
         <v>0</v>
       </c>
       <c r="Q55" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R55" s="1">
-        <v>664.0</v>
+        <v>432.0</v>
       </c>
       <c r="S55" s="1">
-        <v>697439.0</v>
+        <v>554729.0</v>
       </c>
       <c r="T55" s="1">
-        <v>162927364.0</v>
+        <v>96089496.0</v>
       </c>
       <c r="U55" s="1">
-        <v>1051279.0</v>
+        <v>776230.0</v>
       </c>
       <c r="V55" s="1">
-        <v>965009</v>
+        <v>781651</v>
       </c>
       <c r="X55" t="b">
         <v>0</v>
       </c>
       <c r="Y55" t="s">
-        <v>831</v>
+        <v>432</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>827</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="B56" t="s">
         <v>73</v>
@@ -55916,81 +56033,48 @@
         <v>74</v>
       </c>
       <c r="D56" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E56" t="s">
-        <v>110</v>
+        <v>195</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
       </c>
       <c r="G56" s="1">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I56" s="4">
-        <v>46314.354537037034</v>
+        <v>46314.69179398148</v>
       </c>
       <c r="J56" s="4">
-        <v>46314.44809027778</v>
-      </c>
-      <c r="K56" s="3">
-        <v>108.24491666666667</v>
-      </c>
-      <c r="L56" s="2">
-        <v>13.553072</v>
-      </c>
-      <c r="M56" s="2">
-        <v>13.553072</v>
-      </c>
-      <c r="N56" s="2">
-        <v>0</v>
-      </c>
-      <c r="O56" s="1">
-        <v>321</v>
-      </c>
-      <c r="P56" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q56" s="1">
-        <v>1</v>
-      </c>
-      <c r="R56" s="1">
-        <v>934.0</v>
-      </c>
-      <c r="S56" s="1">
-        <v>907702.0</v>
-      </c>
-      <c r="T56" s="1">
-        <v>203600498.0</v>
-      </c>
-      <c r="U56" s="1">
-        <v>1342643.0</v>
-      </c>
-      <c r="V56" s="1">
-        <v>964812</v>
+        <v>46314.70092592593</v>
       </c>
       <c r="X56" t="b">
         <v>0</v>
       </c>
       <c r="Y56" t="s">
-        <v>833</v>
+        <v>196</v>
+      </c>
+      <c r="Z56" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>834</v>
+        <v>830</v>
       </c>
       <c r="B57" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C57" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D57" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" t="s">
         <v>110</v>
@@ -55999,104 +56083,143 @@
         <v>1</v>
       </c>
       <c r="G57" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H57" t="b">
         <v>0</v>
       </c>
       <c r="I57" s="4">
-        <v>46315.19510416667</v>
+        <v>46314.25201388889</v>
       </c>
       <c r="J57" s="4">
-        <v>46315.23210648148</v>
+        <v>46314.32546296297</v>
       </c>
       <c r="K57" s="3">
-        <v>47.0307</v>
+        <v>95.18496666666667</v>
       </c>
       <c r="L57" s="2">
-        <v>7.028553</v>
+        <v>10.606161</v>
       </c>
       <c r="M57" s="2">
-        <v>2.251192</v>
+        <v>10.606161</v>
       </c>
       <c r="N57" s="2">
-        <v>4.777361</v>
+        <v>0</v>
       </c>
       <c r="O57" s="1">
-        <v>14</v>
+        <v>335</v>
       </c>
       <c r="P57" s="1">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q57" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R57" s="1">
-        <v>671679.0</v>
+        <v>664.0</v>
       </c>
       <c r="S57" s="1">
-        <v>201151.0</v>
+        <v>697439.0</v>
       </c>
       <c r="T57" s="1">
-        <v>21039932.0</v>
+        <v>162927364.0</v>
       </c>
       <c r="U57" s="1">
-        <v>111024.0</v>
+        <v>1051279.0</v>
       </c>
       <c r="V57" s="1">
-        <v>111026</v>
-      </c>
-      <c r="W57" s="1">
-        <v>186027</v>
+        <v>965009</v>
       </c>
       <c r="X57" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Y57" t="s">
+        <v>831</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="B58" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C58" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D58" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" t="s">
-        <v>787</v>
+        <v>110</v>
       </c>
       <c r="F58" t="b">
         <v>0</v>
       </c>
       <c r="G58" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" s="4">
-        <v>46315.23091435185</v>
+        <v>46314.354537037034</v>
+      </c>
+      <c r="J58" s="4">
+        <v>46314.44809027778</v>
+      </c>
+      <c r="K58" s="3">
+        <v>108.24491666666667</v>
+      </c>
+      <c r="L58" s="2">
+        <v>13.553072</v>
+      </c>
+      <c r="M58" s="2">
+        <v>13.553072</v>
+      </c>
+      <c r="N58" s="2">
+        <v>0</v>
+      </c>
+      <c r="O58" s="1">
+        <v>321</v>
+      </c>
+      <c r="P58" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="1">
+        <v>1</v>
+      </c>
+      <c r="R58" s="1">
+        <v>934.0</v>
+      </c>
+      <c r="S58" s="1">
+        <v>907702.0</v>
+      </c>
+      <c r="T58" s="1">
+        <v>203600498.0</v>
+      </c>
+      <c r="U58" s="1">
+        <v>1342643.0</v>
+      </c>
+      <c r="V58" s="1">
+        <v>964812</v>
       </c>
       <c r="X58" t="b">
         <v>0</v>
       </c>
       <c r="Y58" t="s">
-        <v>788</v>
+        <v>833</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="B59" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C59" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D59" s="1">
         <v>1</v>
@@ -56114,49 +56237,49 @@
         <v>0</v>
       </c>
       <c r="I59" s="4">
-        <v>46315.195289351854</v>
+        <v>46315.19510416667</v>
       </c>
       <c r="J59" s="4">
-        <v>46315.22857638889</v>
+        <v>46315.23210648148</v>
       </c>
       <c r="K59" s="3">
-        <v>41.971066666666665</v>
+        <v>47.0307</v>
       </c>
       <c r="L59" s="2">
-        <v>10.33528</v>
+        <v>7.028553</v>
       </c>
       <c r="M59" s="2">
-        <v>8.729592</v>
+        <v>2.251192</v>
       </c>
       <c r="N59" s="2">
-        <v>1.605688</v>
+        <v>4.777361</v>
       </c>
       <c r="O59" s="1">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="P59" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q59" s="1">
         <v>0</v>
       </c>
       <c r="R59" s="1">
-        <v>236477.0</v>
+        <v>671679.0</v>
       </c>
       <c r="S59" s="1">
-        <v>202289.0</v>
+        <v>201151.0</v>
       </c>
       <c r="T59" s="1">
-        <v>23194760.0</v>
+        <v>21039932.0</v>
       </c>
       <c r="U59" s="1">
-        <v>288791.0</v>
+        <v>111024.0</v>
       </c>
       <c r="V59" s="1">
-        <v>294098</v>
+        <v>111026</v>
       </c>
       <c r="W59" s="1">
-        <v>126892</v>
+        <v>186027</v>
       </c>
       <c r="X59" t="b">
         <v>1</v>
@@ -56164,37 +56287,372 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="B60" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D60" s="1">
         <v>2</v>
       </c>
       <c r="E60" t="s">
-        <v>787</v>
+        <v>110</v>
       </c>
       <c r="F60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H60" t="b">
         <v>0</v>
       </c>
       <c r="I60" s="4">
+        <v>46315.23091435185</v>
+      </c>
+      <c r="J60" s="4">
+        <v>46315.28097222222</v>
+      </c>
+      <c r="K60" s="3">
+        <v>65.92375</v>
+      </c>
+      <c r="L60" s="2">
+        <v>7.904781</v>
+      </c>
+      <c r="M60" s="2">
+        <v>3.872107</v>
+      </c>
+      <c r="N60" s="2">
+        <v>4.032674</v>
+      </c>
+      <c r="O60" s="1">
+        <v>14</v>
+      </c>
+      <c r="P60" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q60" s="1">
+        <v>0</v>
+      </c>
+      <c r="R60" s="1">
+        <v>680425.0</v>
+      </c>
+      <c r="S60" s="1">
+        <v>214328.0</v>
+      </c>
+      <c r="T60" s="1">
+        <v>18129177.0</v>
+      </c>
+      <c r="U60" s="1">
+        <v>162920.0</v>
+      </c>
+      <c r="V60" s="1">
+        <v>168227</v>
+      </c>
+      <c r="W60" s="1">
+        <v>131067</v>
+      </c>
+      <c r="X60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>836</v>
+      </c>
+      <c r="B61" t="s">
+        <v>79</v>
+      </c>
+      <c r="C61" t="s">
+        <v>80</v>
+      </c>
+      <c r="D61" s="1">
+        <v>3</v>
+      </c>
+      <c r="E61" t="s">
+        <v>110</v>
+      </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
+      <c r="G61" s="1">
+        <v>1</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" s="4">
+        <v>46315.263287037036</v>
+      </c>
+      <c r="J61" s="4">
+        <v>46315.304560185185</v>
+      </c>
+      <c r="K61" s="3">
+        <v>53.20843333333333</v>
+      </c>
+      <c r="L61" s="2">
+        <v>8.404477</v>
+      </c>
+      <c r="M61" s="2">
+        <v>3.100943</v>
+      </c>
+      <c r="N61" s="2">
+        <v>5.303534</v>
+      </c>
+      <c r="O61" s="1">
+        <v>11</v>
+      </c>
+      <c r="P61" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q61" s="1">
+        <v>0</v>
+      </c>
+      <c r="R61" s="1">
+        <v>739138.0</v>
+      </c>
+      <c r="S61" s="1">
+        <v>218134.0</v>
+      </c>
+      <c r="T61" s="1">
+        <v>26303334.0</v>
+      </c>
+      <c r="U61" s="1">
+        <v>141014.0</v>
+      </c>
+      <c r="V61" s="1">
+        <v>146321</v>
+      </c>
+      <c r="W61" s="1">
+        <v>131153</v>
+      </c>
+      <c r="X61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>837</v>
+      </c>
+      <c r="B62" t="s">
+        <v>81</v>
+      </c>
+      <c r="C62" t="s">
+        <v>82</v>
+      </c>
+      <c r="D62" s="1">
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
+        <v>110</v>
+      </c>
+      <c r="F62" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" s="4">
+        <v>46315.195289351854</v>
+      </c>
+      <c r="J62" s="4">
+        <v>46315.22857638889</v>
+      </c>
+      <c r="K62" s="3">
+        <v>41.971066666666665</v>
+      </c>
+      <c r="L62" s="2">
+        <v>10.33528</v>
+      </c>
+      <c r="M62" s="2">
+        <v>8.729592</v>
+      </c>
+      <c r="N62" s="2">
+        <v>1.605688</v>
+      </c>
+      <c r="O62" s="1">
+        <v>99</v>
+      </c>
+      <c r="P62" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q62" s="1">
+        <v>0</v>
+      </c>
+      <c r="R62" s="1">
+        <v>236477.0</v>
+      </c>
+      <c r="S62" s="1">
+        <v>202289.0</v>
+      </c>
+      <c r="T62" s="1">
+        <v>23194760.0</v>
+      </c>
+      <c r="U62" s="1">
+        <v>288791.0</v>
+      </c>
+      <c r="V62" s="1">
+        <v>294098</v>
+      </c>
+      <c r="W62" s="1">
+        <v>126892</v>
+      </c>
+      <c r="X62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>838</v>
+      </c>
+      <c r="B63" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" t="s">
+        <v>82</v>
+      </c>
+      <c r="D63" s="1">
+        <v>2</v>
+      </c>
+      <c r="E63" t="s">
+        <v>110</v>
+      </c>
+      <c r="F63" t="b">
+        <v>1</v>
+      </c>
+      <c r="G63" s="1">
+        <v>1</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" s="4">
         <v>46315.232256944444</v>
       </c>
-      <c r="X60" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y60" t="s">
-        <v>788</v>
+      <c r="J63" s="4">
+        <v>46315.258472222224</v>
+      </c>
+      <c r="K63" s="3">
+        <v>31.6082</v>
+      </c>
+      <c r="L63" s="2">
+        <v>10.422728</v>
+      </c>
+      <c r="M63" s="2">
+        <v>9.554582</v>
+      </c>
+      <c r="N63" s="2">
+        <v>0.868146</v>
+      </c>
+      <c r="O63" s="1">
+        <v>108</v>
+      </c>
+      <c r="P63" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q63" s="1">
+        <v>0</v>
+      </c>
+      <c r="R63" s="1">
+        <v>117674.0</v>
+      </c>
+      <c r="S63" s="1">
+        <v>194292.0</v>
+      </c>
+      <c r="T63" s="1">
+        <v>22870850.0</v>
+      </c>
+      <c r="U63" s="1">
+        <v>295021.0</v>
+      </c>
+      <c r="V63" s="1">
+        <v>300328</v>
+      </c>
+      <c r="W63" s="1">
+        <v>111622</v>
+      </c>
+      <c r="X63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>839</v>
+      </c>
+      <c r="B64" t="s">
+        <v>81</v>
+      </c>
+      <c r="C64" t="s">
+        <v>82</v>
+      </c>
+      <c r="D64" s="1">
+        <v>3</v>
+      </c>
+      <c r="E64" t="s">
+        <v>110</v>
+      </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" s="1">
+        <v>1</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" s="4">
+        <v>46315.28113425926</v>
+      </c>
+      <c r="J64" s="4">
+        <v>46315.31790509259</v>
+      </c>
+      <c r="K64" s="3">
+        <v>46.82698333333334</v>
+      </c>
+      <c r="L64" s="2">
+        <v>12.894339</v>
+      </c>
+      <c r="M64" s="2">
+        <v>11.423216</v>
+      </c>
+      <c r="N64" s="2">
+        <v>1.471124</v>
+      </c>
+      <c r="O64" s="1">
+        <v>16</v>
+      </c>
+      <c r="P64" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q64" s="1">
+        <v>0</v>
+      </c>
+      <c r="R64" s="1">
+        <v>224848.0</v>
+      </c>
+      <c r="S64" s="1">
+        <v>229914.0</v>
+      </c>
+      <c r="T64" s="1">
+        <v>30561675.0</v>
+      </c>
+      <c r="U64" s="1">
+        <v>344432.0</v>
+      </c>
+      <c r="V64" s="1">
+        <v>349739</v>
+      </c>
+      <c r="W64" s="1">
+        <v>123693</v>
+      </c>
+      <c r="X64" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Task 4 results: add A26 and A30 (6 runs, all passed)
A26 (solo GPT-6.1 Sol) is the cheapest Task 4 arm at 1.68 USD per pass; A30
costs 3.41. Five of the six runs needed a second round, each for missing
report sections only. Charts redrawn and workbook re-exported.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/results/experiment-a-results.xlsx
+++ b/docs/results/experiment-a-results.xlsx
@@ -19,12 +19,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4432" uniqueCount="1172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4430" uniqueCount="1170">
   <si>
     <t xml:space="preserve">Experiment results workbook</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated: 2026-10-21 13:32:46 UTC</t>
+    <t xml:space="preserve">Generated: 2026-10-21 14:28:55 UTC</t>
   </si>
   <si>
     <t xml:space="preserve">Runs directory: /workspace/agent-experiments-matrix</t>
@@ -39,7 +39,7 @@
     <t xml:space="preserve">Statuses dropped: accounting_error, cli_error, running, stopped, usage_limit, validation_error</t>
   </si>
   <si>
-    <t xml:space="preserve">Attempts per task: task1: 310 of 321 attempts in the results; task2: 293 of 309 attempts in the results; task3: 191 of 244 attempts in the results; task4: 18 of 75 attempts in the results</t>
+    <t xml:space="preserve">Attempts per task: task1: 310 of 321 attempts in the results; task2: 293 of 309 attempts in the results; task3: 191 of 244 attempts in the results; task4: 24 of 75 attempts in the results</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -3514,12 +3514,6 @@
   </si>
   <si>
     <t xml:space="preserve">aab865b8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">running</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dropped status: running</t>
   </si>
   <si>
     <t xml:space="preserve">b1c278ba</t>
@@ -3808,8 +3802,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC7" totalsRowShown="0">
-  <autoFilter ref="A1:AC7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Summary_T4" displayName="Summary_T4" ref="A1:AC9" totalsRowShown="0">
+  <autoFilter ref="A1:AC9"/>
   <tableColumns count="29">
     <tableColumn id="1" name="Arm"/>
     <tableColumn id="2" name="Description"/>
@@ -75157,7 +75151,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC7"/>
+  <dimension ref="A1:AC9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -75794,6 +75788,172 @@
       </c>
       <c r="AC7" s="3">
         <v>173.813</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1.680172</v>
+      </c>
+      <c r="G8" s="2">
+        <v>5.040516</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1.504043</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1.729886</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1.806587</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.3025439999999999</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>1.729886</v>
+      </c>
+      <c r="N8" s="3">
+        <v>26.2104</v>
+      </c>
+      <c r="O8" s="3">
+        <v>26.619233333333334</v>
+      </c>
+      <c r="P8" s="3">
+        <v>31.24798333333333</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>70</v>
+      </c>
+      <c r="R8" s="1">
+        <v>83</v>
+      </c>
+      <c r="S8" s="1">
+        <v>0</v>
+      </c>
+      <c r="T8" s="1">
+        <v>0</v>
+      </c>
+      <c r="U8" s="1">
+        <v>1</v>
+      </c>
+      <c r="V8" s="1">
+        <v>2</v>
+      </c>
+      <c r="W8" s="1">
+        <v>2</v>
+      </c>
+      <c r="X8" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="3">
+        <v>164.074</v>
+      </c>
+      <c r="AA8" s="3">
+        <v>179.842</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="1">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2">
+        <v>3.4118209999999998</v>
+      </c>
+      <c r="G9" s="2">
+        <v>10.235463</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2.464966</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3.360695</v>
+      </c>
+      <c r="J9" s="2">
+        <v>4.409802</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1.944836</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>3.360694</v>
+      </c>
+      <c r="N9" s="3">
+        <v>27.742283333333333</v>
+      </c>
+      <c r="O9" s="3">
+        <v>36.228966666666665</v>
+      </c>
+      <c r="P9" s="3">
+        <v>45.526716666666665</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>152</v>
+      </c>
+      <c r="R9" s="1">
+        <v>225</v>
+      </c>
+      <c r="S9" s="1">
+        <v>6</v>
+      </c>
+      <c r="T9" s="1">
+        <v>8</v>
+      </c>
+      <c r="U9" s="1">
+        <v>2</v>
+      </c>
+      <c r="V9" s="1">
+        <v>2</v>
+      </c>
+      <c r="W9" s="1">
+        <v>3</v>
+      </c>
+      <c r="X9" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>2</v>
+      </c>
+      <c r="Z9" s="3">
+        <v>132.275</v>
+      </c>
+      <c r="AA9" s="3">
+        <v>219.284</v>
+      </c>
+      <c r="AB9" s="3">
+        <v>172.614</v>
+      </c>
+      <c r="AC9" s="3">
+        <v>179.94</v>
       </c>
     </row>
   </sheetData>
@@ -81129,13 +81289,13 @@
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G71" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H71" t="b">
         <v>0</v>
@@ -81143,16 +81303,52 @@
       <c r="I71" s="4">
         <v>46316.56350694445</v>
       </c>
+      <c r="J71" s="4">
+        <v>46316.58571759259</v>
+      </c>
+      <c r="K71" s="3">
+        <v>26.2104</v>
+      </c>
+      <c r="L71" s="2">
+        <v>1.729886</v>
+      </c>
+      <c r="M71" s="2">
+        <v>0</v>
+      </c>
+      <c r="N71" s="2">
+        <v>1.729886</v>
+      </c>
+      <c r="O71" s="1">
+        <v>75</v>
+      </c>
+      <c r="P71" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="1">
+        <v>0</v>
+      </c>
+      <c r="R71" s="1">
+        <v>180994.0</v>
+      </c>
+      <c r="S71" s="1">
+        <v>55826.0</v>
+      </c>
+      <c r="T71" s="1">
+        <v>8096384.0</v>
+      </c>
+      <c r="U71" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V71" s="1">
+        <v>167796</v>
+      </c>
       <c r="X71" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y71" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="B72" t="s">
         <v>89</v>
@@ -81164,13 +81360,13 @@
         <v>2</v>
       </c>
       <c r="E72" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G72" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H72" t="b">
         <v>0</v>
@@ -81178,16 +81374,52 @@
       <c r="I72" s="4">
         <v>46316.56386574074</v>
       </c>
+      <c r="J72" s="4">
+        <v>46316.593773148146</v>
+      </c>
+      <c r="K72" s="3">
+        <v>31.24798333333333</v>
+      </c>
+      <c r="L72" s="2">
+        <v>1.806587</v>
+      </c>
+      <c r="M72" s="2">
+        <v>0</v>
+      </c>
+      <c r="N72" s="2">
+        <v>1.806587</v>
+      </c>
+      <c r="O72" s="1">
+        <v>83</v>
+      </c>
+      <c r="P72" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="1">
+        <v>0</v>
+      </c>
+      <c r="R72" s="1">
+        <v>123693.0</v>
+      </c>
+      <c r="S72" s="1">
+        <v>59851.0</v>
+      </c>
+      <c r="T72" s="1">
+        <v>9606912.0</v>
+      </c>
+      <c r="U72" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V72" s="1">
+        <v>179842</v>
+      </c>
       <c r="X72" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y72" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="B73" t="s">
         <v>89</v>
@@ -81199,13 +81431,13 @@
         <v>3</v>
       </c>
       <c r="E73" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G73" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H73" t="b">
         <v>0</v>
@@ -81213,16 +81445,52 @@
       <c r="I73" s="4">
         <v>46316.564247685186</v>
       </c>
+      <c r="J73" s="4">
+        <v>46316.590787037036</v>
+      </c>
+      <c r="K73" s="3">
+        <v>26.619233333333334</v>
+      </c>
+      <c r="L73" s="2">
+        <v>1.504043</v>
+      </c>
+      <c r="M73" s="2">
+        <v>0</v>
+      </c>
+      <c r="N73" s="2">
+        <v>1.504043</v>
+      </c>
+      <c r="O73" s="1">
+        <v>70</v>
+      </c>
+      <c r="P73" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="1">
+        <v>0</v>
+      </c>
+      <c r="R73" s="1">
+        <v>115148.0</v>
+      </c>
+      <c r="S73" s="1">
+        <v>54183.0</v>
+      </c>
+      <c r="T73" s="1">
+        <v>7319168.0</v>
+      </c>
+      <c r="U73" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V73" s="1">
+        <v>164074</v>
+      </c>
       <c r="X73" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y73" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="B74" t="s">
         <v>97</v>
@@ -81234,13 +81502,13 @@
         <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G74" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H74" t="b">
         <v>0</v>
@@ -81248,16 +81516,55 @@
       <c r="I74" s="4">
         <v>46316.56369212963</v>
       </c>
+      <c r="J74" s="4">
+        <v>46316.603414351855</v>
+      </c>
+      <c r="K74" s="3">
+        <v>45.526716666666665</v>
+      </c>
+      <c r="L74" s="2">
+        <v>4.409802</v>
+      </c>
+      <c r="M74" s="2">
+        <v>0</v>
+      </c>
+      <c r="N74" s="2">
+        <v>4.409801</v>
+      </c>
+      <c r="O74" s="1">
+        <v>225</v>
+      </c>
+      <c r="P74" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q74" s="1">
+        <v>1</v>
+      </c>
+      <c r="R74" s="1">
+        <v>955472.0</v>
+      </c>
+      <c r="S74" s="1">
+        <v>255732.0</v>
+      </c>
+      <c r="T74" s="1">
+        <v>69593984.0</v>
+      </c>
+      <c r="U74" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V74" s="1">
+        <v>219284</v>
+      </c>
+      <c r="W74" s="1">
+        <v>172614</v>
+      </c>
       <c r="X74" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y74" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B75" t="s">
         <v>97</v>
@@ -81269,13 +81576,13 @@
         <v>2</v>
       </c>
       <c r="E75" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H75" t="b">
         <v>0</v>
@@ -81283,16 +81590,55 @@
       <c r="I75" s="4">
         <v>46316.5640625</v>
       </c>
+      <c r="J75" s="4">
+        <v>46316.59721064815</v>
+      </c>
+      <c r="K75" s="3">
+        <v>36.228966666666665</v>
+      </c>
+      <c r="L75" s="2">
+        <v>3.360695</v>
+      </c>
+      <c r="M75" s="2">
+        <v>0</v>
+      </c>
+      <c r="N75" s="2">
+        <v>3.360694</v>
+      </c>
+      <c r="O75" s="1">
+        <v>183</v>
+      </c>
+      <c r="P75" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q75" s="1">
+        <v>1</v>
+      </c>
+      <c r="R75" s="1">
+        <v>1035434.0</v>
+      </c>
+      <c r="S75" s="1">
+        <v>217545.0</v>
+      </c>
+      <c r="T75" s="1">
+        <v>67784448.0</v>
+      </c>
+      <c r="U75" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V75" s="1">
+        <v>185097</v>
+      </c>
+      <c r="W75" s="1">
+        <v>179940</v>
+      </c>
       <c r="X75" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y75" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="B76" t="s">
         <v>97</v>
@@ -81304,13 +81650,13 @@
         <v>3</v>
       </c>
       <c r="E76" t="s">
-        <v>1165</v>
+        <v>130</v>
       </c>
       <c r="F76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H76" t="b">
         <v>0</v>
@@ -81318,11 +81664,50 @@
       <c r="I76" s="4">
         <v>46316.564421296294</v>
       </c>
+      <c r="J76" s="4">
+        <v>46316.59168981481</v>
+      </c>
+      <c r="K76" s="3">
+        <v>27.742283333333333</v>
+      </c>
+      <c r="L76" s="2">
+        <v>2.464966</v>
+      </c>
+      <c r="M76" s="2">
+        <v>0</v>
+      </c>
+      <c r="N76" s="2">
+        <v>2.464966</v>
+      </c>
+      <c r="O76" s="1">
+        <v>152</v>
+      </c>
+      <c r="P76" s="1">
+        <v>8</v>
+      </c>
+      <c r="Q76" s="1">
+        <v>2</v>
+      </c>
+      <c r="R76" s="1">
+        <v>1129960.0</v>
+      </c>
+      <c r="S76" s="1">
+        <v>259145.0</v>
+      </c>
+      <c r="T76" s="1">
+        <v>72234496.0</v>
+      </c>
+      <c r="U76" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="V76" s="1">
+        <v>132275</v>
+      </c>
+      <c r="W76" s="1">
+        <v>178941</v>
+      </c>
       <c r="X76" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y76" t="s">
-        <v>1166</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>